<commit_message>
data(jpy): daily refresh 2026-10-14T08:59Z
</commit_message>
<xml_diff>
--- a/history/jpy/mei_latest.xlsx
+++ b/history/jpy/mei_latest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{45EDF400-56B6-486C-9433-93D2286D41A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF7CB05A-4A63-41A8-919E-1EB1A17E14D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">mei!$A$1:$G$369</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1357,7 +1357,7 @@
   <sheetData>
     <row r="3" spans="1:8" ht="18.75" customHeight="1">
       <c r="A3" s="50">
-        <v>46295</v>
+        <v>46304</v>
       </c>
       <c r="B3" s="50"/>
       <c r="C3" s="50"/>
@@ -1368,7 +1368,7 @@
     </row>
     <row r="4" spans="1:8" ht="18.75" customHeight="1">
       <c r="A4" s="51">
-        <v>46295</v>
+        <v>46304</v>
       </c>
       <c r="B4" s="51"/>
       <c r="C4" s="51"/>
@@ -1386,10 +1386,10 @@
     </row>
     <row r="7" spans="1:8" ht="18.75" customHeight="1">
       <c r="B7" s="12">
-        <v>46297</v>
+        <v>46309</v>
       </c>
       <c r="F7" s="29">
-        <v>46297</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18.75" customHeight="1">
@@ -1459,10 +1459,10 @@
         <v>18</v>
       </c>
       <c r="D16" s="48">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E16" s="49">
-        <v>12234</v>
+        <v>8331</v>
       </c>
       <c r="F16" s="33"/>
       <c r="G16" s="2"/>
@@ -1474,10 +1474,10 @@
         <v>29</v>
       </c>
       <c r="D17" s="42">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E17" s="43">
-        <v>7884</v>
+        <v>6043</v>
       </c>
       <c r="F17" s="33"/>
       <c r="G17" s="2"/>
@@ -1487,10 +1487,10 @@
       <c r="B18" s="1"/>
       <c r="C18" s="41"/>
       <c r="D18" s="42">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E18" s="43">
-        <v>6043</v>
+        <v>5522</v>
       </c>
       <c r="F18" s="33"/>
       <c r="G18" s="2"/>
@@ -1500,10 +1500,10 @@
       <c r="B19" s="1"/>
       <c r="C19" s="41"/>
       <c r="D19" s="42">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E19" s="43">
-        <v>5522</v>
+        <v>7588</v>
       </c>
       <c r="F19" s="33"/>
       <c r="G19" s="2"/>
@@ -1513,10 +1513,10 @@
       <c r="B20" s="1"/>
       <c r="C20" s="41"/>
       <c r="D20" s="42">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E20" s="43">
-        <v>7588</v>
+        <v>1613</v>
       </c>
       <c r="F20" s="33"/>
       <c r="G20" s="2"/>
@@ -1526,10 +1526,10 @@
       <c r="B21" s="1"/>
       <c r="C21" s="41"/>
       <c r="D21" s="42">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E21" s="43">
-        <v>1353</v>
+        <v>6169</v>
       </c>
       <c r="F21" s="33"/>
       <c r="G21" s="2"/>
@@ -1539,10 +1539,10 @@
       <c r="B22" s="1"/>
       <c r="C22" s="41"/>
       <c r="D22" s="42">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E22" s="43">
-        <v>6167</v>
+        <v>2296</v>
       </c>
       <c r="F22" s="33"/>
       <c r="G22" s="2"/>
@@ -1552,10 +1552,10 @@
       <c r="B23" s="1"/>
       <c r="C23" s="41"/>
       <c r="D23" s="42">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E23" s="43">
-        <v>2296</v>
+        <v>12370</v>
       </c>
       <c r="F23" s="33"/>
       <c r="G23" s="2"/>
@@ -1565,10 +1565,10 @@
       <c r="B24" s="1"/>
       <c r="C24" s="41"/>
       <c r="D24" s="42">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E24" s="43">
-        <v>12370</v>
+        <v>4199</v>
       </c>
       <c r="F24" s="33"/>
       <c r="G24" s="2"/>
@@ -1578,10 +1578,10 @@
       <c r="B25" s="1"/>
       <c r="C25" s="41"/>
       <c r="D25" s="42">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E25" s="43">
-        <v>4199</v>
+        <v>13323</v>
       </c>
       <c r="F25" s="33"/>
       <c r="G25" s="2"/>
@@ -1591,10 +1591,10 @@
       <c r="B26" s="1"/>
       <c r="C26" s="41"/>
       <c r="D26" s="42">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E26" s="43">
-        <v>13323</v>
+        <v>6543</v>
       </c>
       <c r="F26" s="33"/>
       <c r="G26" s="2"/>
@@ -1604,10 +1604,10 @@
       <c r="B27" s="1"/>
       <c r="C27" s="41"/>
       <c r="D27" s="42">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E27" s="43">
-        <v>6543</v>
+        <v>6417</v>
       </c>
       <c r="F27" s="33"/>
       <c r="G27" s="2"/>
@@ -1617,10 +1617,10 @@
       <c r="B28" s="1"/>
       <c r="C28" s="41"/>
       <c r="D28" s="42">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="E28" s="43">
-        <v>6260</v>
+        <v>6131</v>
       </c>
       <c r="F28" s="33"/>
       <c r="G28" s="2"/>
@@ -1630,10 +1630,10 @@
       <c r="B29" s="1"/>
       <c r="C29" s="41"/>
       <c r="D29" s="42">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E29" s="43">
-        <v>6108</v>
+        <v>1940</v>
       </c>
       <c r="F29" s="33"/>
       <c r="G29" s="2"/>
@@ -1643,10 +1643,10 @@
       <c r="B30" s="1"/>
       <c r="C30" s="41"/>
       <c r="D30" s="42">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E30" s="43">
-        <v>1867</v>
+        <v>4576</v>
       </c>
       <c r="F30" s="33"/>
       <c r="G30" s="2"/>
@@ -1656,10 +1656,10 @@
       <c r="B31" s="1"/>
       <c r="C31" s="41"/>
       <c r="D31" s="42">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E31" s="43">
-        <v>4476</v>
+        <v>8368</v>
       </c>
       <c r="F31" s="33"/>
       <c r="G31" s="2"/>
@@ -1669,10 +1669,10 @@
       <c r="B32" s="1"/>
       <c r="C32" s="41"/>
       <c r="D32" s="42">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="E32" s="43">
-        <v>7919</v>
+        <v>2046</v>
       </c>
       <c r="F32" s="33"/>
       <c r="G32" s="2"/>
@@ -1682,10 +1682,10 @@
       <c r="B33" s="1"/>
       <c r="C33" s="41"/>
       <c r="D33" s="42">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E33" s="43">
-        <v>2046</v>
+        <v>4775</v>
       </c>
       <c r="F33" s="33"/>
       <c r="G33" s="2"/>
@@ -1695,10 +1695,10 @@
       <c r="B34" s="1"/>
       <c r="C34" s="41"/>
       <c r="D34" s="42">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="E34" s="43">
-        <v>4037</v>
+        <v>2585</v>
       </c>
       <c r="F34" s="33"/>
       <c r="G34" s="2"/>
@@ -1708,10 +1708,10 @@
       <c r="B35" s="1"/>
       <c r="C35" s="41"/>
       <c r="D35" s="42">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E35" s="43">
-        <v>2492</v>
+        <v>695</v>
       </c>
       <c r="F35" s="33"/>
       <c r="G35" s="2"/>
@@ -1721,10 +1721,10 @@
       <c r="B36" s="1"/>
       <c r="C36" s="41"/>
       <c r="D36" s="42">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E36" s="43">
-        <v>176</v>
+        <v>76</v>
       </c>
       <c r="F36" s="33"/>
       <c r="G36" s="2"/>
@@ -1734,10 +1734,10 @@
       <c r="B37" s="1"/>
       <c r="C37" s="41"/>
       <c r="D37" s="42">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E37" s="43">
-        <v>76</v>
+        <v>933</v>
       </c>
       <c r="F37" s="33"/>
       <c r="G37" s="2"/>
@@ -1745,12 +1745,12 @@
     </row>
     <row r="38" spans="2:8" ht="18.75" customHeight="1">
       <c r="B38" s="1"/>
-      <c r="C38" s="60"/>
-      <c r="D38" s="61">
-        <v>487</v>
-      </c>
-      <c r="E38" s="64">
-        <v>933</v>
+      <c r="C38" s="41"/>
+      <c r="D38" s="42">
+        <v>488</v>
+      </c>
+      <c r="E38" s="43">
+        <v>154</v>
       </c>
       <c r="F38" s="33"/>
       <c r="G38" s="2"/>
@@ -1758,14 +1758,12 @@
     </row>
     <row r="39" spans="2:8" ht="18.75" customHeight="1">
       <c r="B39" s="1"/>
-      <c r="C39" s="62" t="s">
-        <v>19</v>
-      </c>
-      <c r="D39" s="63">
-        <v>150</v>
-      </c>
-      <c r="E39" s="65">
-        <v>57060</v>
+      <c r="C39" s="60"/>
+      <c r="D39" s="61">
+        <v>489</v>
+      </c>
+      <c r="E39" s="64">
+        <v>862</v>
       </c>
       <c r="F39" s="33"/>
       <c r="G39" s="2"/>
@@ -1773,14 +1771,14 @@
     </row>
     <row r="40" spans="2:8" ht="18.75" customHeight="1">
       <c r="B40" s="1"/>
-      <c r="C40" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="D40" s="42">
-        <v>151</v>
-      </c>
-      <c r="E40" s="43">
-        <v>36566</v>
+      <c r="C40" s="62" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="63">
+        <v>150</v>
+      </c>
+      <c r="E40" s="65">
+        <v>57060</v>
       </c>
       <c r="F40" s="33"/>
       <c r="G40" s="2"/>
@@ -1788,12 +1786,14 @@
     </row>
     <row r="41" spans="2:8" ht="18.75" customHeight="1">
       <c r="B41" s="1"/>
-      <c r="C41" s="41"/>
+      <c r="C41" s="41" t="s">
+        <v>30</v>
+      </c>
       <c r="D41" s="42">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E41" s="43">
-        <v>18662</v>
+        <v>36566</v>
       </c>
       <c r="F41" s="33"/>
       <c r="G41" s="2"/>
@@ -1803,10 +1803,10 @@
       <c r="B42" s="1"/>
       <c r="C42" s="41"/>
       <c r="D42" s="42">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E42" s="43">
-        <v>65018</v>
+        <v>18662</v>
       </c>
       <c r="F42" s="33"/>
       <c r="G42" s="2"/>
@@ -1816,10 +1816,10 @@
       <c r="B43" s="1"/>
       <c r="C43" s="41"/>
       <c r="D43" s="42">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E43" s="43">
-        <v>57072</v>
+        <v>65018</v>
       </c>
       <c r="F43" s="33"/>
       <c r="G43" s="2"/>
@@ -1829,10 +1829,10 @@
       <c r="B44" s="1"/>
       <c r="C44" s="41"/>
       <c r="D44" s="42">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E44" s="43">
-        <v>21500</v>
+        <v>57072</v>
       </c>
       <c r="F44" s="33"/>
       <c r="G44" s="2"/>
@@ -1842,10 +1842,10 @@
       <c r="B45" s="1"/>
       <c r="C45" s="41"/>
       <c r="D45" s="42">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E45" s="43">
-        <v>44981</v>
+        <v>21500</v>
       </c>
       <c r="F45" s="33"/>
       <c r="G45" s="2"/>
@@ -1855,10 +1855,10 @@
       <c r="B46" s="1"/>
       <c r="C46" s="41"/>
       <c r="D46" s="42">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E46" s="43">
-        <v>18460</v>
+        <v>44981</v>
       </c>
       <c r="F46" s="33"/>
       <c r="G46" s="2"/>
@@ -1868,10 +1868,10 @@
       <c r="B47" s="1"/>
       <c r="C47" s="41"/>
       <c r="D47" s="42">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E47" s="43">
-        <v>40190</v>
+        <v>18470</v>
       </c>
       <c r="F47" s="33"/>
       <c r="G47" s="2"/>
@@ -1881,10 +1881,10 @@
       <c r="B48" s="1"/>
       <c r="C48" s="41"/>
       <c r="D48" s="42">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E48" s="43">
-        <v>17892</v>
+        <v>40190</v>
       </c>
       <c r="F48" s="33"/>
       <c r="G48" s="2"/>
@@ -1894,10 +1894,10 @@
       <c r="B49" s="1"/>
       <c r="C49" s="41"/>
       <c r="D49" s="42">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E49" s="43">
-        <v>18440</v>
+        <v>17892</v>
       </c>
       <c r="F49" s="33"/>
       <c r="G49" s="2"/>
@@ -1907,10 +1907,10 @@
       <c r="B50" s="1"/>
       <c r="C50" s="41"/>
       <c r="D50" s="42">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E50" s="43">
-        <v>17767</v>
+        <v>18440</v>
       </c>
       <c r="F50" s="33"/>
       <c r="G50" s="2"/>
@@ -1920,10 +1920,10 @@
       <c r="B51" s="1"/>
       <c r="C51" s="41"/>
       <c r="D51" s="42">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E51" s="43">
-        <v>18311</v>
+        <v>17767</v>
       </c>
       <c r="F51" s="33"/>
       <c r="G51" s="2"/>
@@ -1933,10 +1933,10 @@
       <c r="B52" s="1"/>
       <c r="C52" s="41"/>
       <c r="D52" s="42">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E52" s="43">
-        <v>45179</v>
+        <v>18311</v>
       </c>
       <c r="F52" s="33"/>
       <c r="G52" s="2"/>
@@ -1946,10 +1946,10 @@
       <c r="B53" s="1"/>
       <c r="C53" s="41"/>
       <c r="D53" s="42">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E53" s="43">
-        <v>15939</v>
+        <v>45179</v>
       </c>
       <c r="F53" s="33"/>
       <c r="G53" s="2"/>
@@ -1959,10 +1959,10 @@
       <c r="B54" s="1"/>
       <c r="C54" s="41"/>
       <c r="D54" s="42">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E54" s="43">
-        <v>14431</v>
+        <v>15939</v>
       </c>
       <c r="F54" s="33"/>
       <c r="G54" s="2"/>
@@ -1972,10 +1972,10 @@
       <c r="B55" s="1"/>
       <c r="C55" s="41"/>
       <c r="D55" s="42">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E55" s="43">
-        <v>10752</v>
+        <v>14455</v>
       </c>
       <c r="F55" s="33"/>
       <c r="G55" s="2"/>
@@ -1985,10 +1985,10 @@
       <c r="B56" s="1"/>
       <c r="C56" s="41"/>
       <c r="D56" s="42">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E56" s="43">
-        <v>9321</v>
+        <v>10785</v>
       </c>
       <c r="F56" s="33"/>
       <c r="G56" s="2"/>
@@ -1998,10 +1998,10 @@
       <c r="B57" s="1"/>
       <c r="C57" s="41"/>
       <c r="D57" s="42">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E57" s="43">
-        <v>13745</v>
+        <v>9335</v>
       </c>
       <c r="F57" s="33"/>
       <c r="G57" s="2"/>
@@ -2011,10 +2011,10 @@
       <c r="B58" s="1"/>
       <c r="C58" s="41"/>
       <c r="D58" s="42">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E58" s="43">
-        <v>14900</v>
+        <v>13758</v>
       </c>
       <c r="F58" s="33"/>
       <c r="G58" s="2"/>
@@ -2024,10 +2024,10 @@
       <c r="B59" s="1"/>
       <c r="C59" s="41"/>
       <c r="D59" s="42">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E59" s="43">
-        <v>16329</v>
+        <v>14905</v>
       </c>
       <c r="F59" s="33"/>
       <c r="G59" s="2"/>
@@ -2037,10 +2037,10 @@
       <c r="B60" s="1"/>
       <c r="C60" s="41"/>
       <c r="D60" s="42">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E60" s="43">
-        <v>20254</v>
+        <v>16329</v>
       </c>
       <c r="F60" s="33"/>
       <c r="G60" s="2"/>
@@ -2050,10 +2050,10 @@
       <c r="B61" s="1"/>
       <c r="C61" s="41"/>
       <c r="D61" s="42">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E61" s="43">
-        <v>18260</v>
+        <v>20254</v>
       </c>
       <c r="F61" s="33"/>
       <c r="G61" s="2"/>
@@ -2063,10 +2063,10 @@
       <c r="B62" s="1"/>
       <c r="C62" s="41"/>
       <c r="D62" s="42">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E62" s="43">
-        <v>13481</v>
+        <v>18260</v>
       </c>
       <c r="F62" s="33"/>
       <c r="G62" s="2"/>
@@ -2076,10 +2076,10 @@
       <c r="B63" s="1"/>
       <c r="C63" s="41"/>
       <c r="D63" s="42">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E63" s="43">
-        <v>24206</v>
+        <v>13481</v>
       </c>
       <c r="F63" s="33"/>
       <c r="G63" s="2"/>
@@ -2089,10 +2089,10 @@
       <c r="B64" s="1"/>
       <c r="C64" s="41"/>
       <c r="D64" s="42">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E64" s="43">
-        <v>9712</v>
+        <v>24206</v>
       </c>
       <c r="F64" s="33"/>
       <c r="G64" s="2"/>
@@ -2102,10 +2102,10 @@
       <c r="B65" s="1"/>
       <c r="C65" s="41"/>
       <c r="D65" s="42">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E65" s="43">
-        <v>6513</v>
+        <v>9712</v>
       </c>
       <c r="F65" s="33"/>
       <c r="G65" s="2"/>
@@ -2115,10 +2115,10 @@
       <c r="B66" s="1"/>
       <c r="C66" s="41"/>
       <c r="D66" s="42">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E66" s="43">
-        <v>5273</v>
+        <v>6513</v>
       </c>
       <c r="F66" s="33"/>
       <c r="G66" s="2"/>
@@ -2128,10 +2128,10 @@
       <c r="B67" s="1"/>
       <c r="C67" s="41"/>
       <c r="D67" s="42">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E67" s="43">
-        <v>22955</v>
+        <v>5273</v>
       </c>
       <c r="F67" s="33"/>
       <c r="G67" s="2"/>
@@ -2141,10 +2141,10 @@
       <c r="B68" s="1"/>
       <c r="C68" s="41"/>
       <c r="D68" s="42">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E68" s="43">
-        <v>9507</v>
+        <v>22955</v>
       </c>
       <c r="F68" s="33"/>
       <c r="G68" s="2"/>
@@ -2154,10 +2154,10 @@
       <c r="B69" s="1"/>
       <c r="C69" s="41"/>
       <c r="D69" s="42">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E69" s="43">
-        <v>6659</v>
+        <v>9507</v>
       </c>
       <c r="F69" s="33"/>
       <c r="G69" s="2"/>
@@ -2167,10 +2167,10 @@
       <c r="B70" s="1"/>
       <c r="C70" s="41"/>
       <c r="D70" s="42">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E70" s="43">
-        <v>9635</v>
+        <v>6659</v>
       </c>
       <c r="F70" s="33"/>
       <c r="G70" s="2"/>
@@ -2180,10 +2180,10 @@
       <c r="B71" s="1"/>
       <c r="C71" s="41"/>
       <c r="D71" s="42">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E71" s="43">
-        <v>2158</v>
+        <v>9635</v>
       </c>
       <c r="F71" s="33"/>
       <c r="G71" s="2"/>
@@ -2193,10 +2193,10 @@
       <c r="B72" s="1"/>
       <c r="C72" s="41"/>
       <c r="D72" s="42">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E72" s="43">
-        <v>12509</v>
+        <v>2158</v>
       </c>
       <c r="F72" s="33"/>
       <c r="G72" s="2"/>
@@ -2206,10 +2206,10 @@
       <c r="B73" s="1"/>
       <c r="C73" s="41"/>
       <c r="D73" s="42">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E73" s="43">
-        <v>1921</v>
+        <v>12509</v>
       </c>
       <c r="F73" s="33"/>
       <c r="G73" s="2"/>
@@ -2219,10 +2219,10 @@
       <c r="B74" s="1"/>
       <c r="C74" s="41"/>
       <c r="D74" s="42">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E74" s="43">
-        <v>5493</v>
+        <v>1921</v>
       </c>
       <c r="F74" s="33"/>
       <c r="G74" s="2"/>
@@ -2232,10 +2232,10 @@
       <c r="B75" s="1"/>
       <c r="C75" s="41"/>
       <c r="D75" s="42">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E75" s="43">
-        <v>1343</v>
+        <v>5493</v>
       </c>
       <c r="F75" s="33"/>
       <c r="G75" s="2"/>
@@ -2243,12 +2243,12 @@
     </row>
     <row r="76" spans="2:8" ht="18.75" customHeight="1">
       <c r="B76" s="1"/>
-      <c r="C76" s="60"/>
-      <c r="D76" s="61">
-        <v>187</v>
-      </c>
-      <c r="E76" s="64">
-        <v>5365</v>
+      <c r="C76" s="41"/>
+      <c r="D76" s="42">
+        <v>186</v>
+      </c>
+      <c r="E76" s="43">
+        <v>1343</v>
       </c>
       <c r="F76" s="33"/>
       <c r="G76" s="2"/>
@@ -2256,14 +2256,12 @@
     </row>
     <row r="77" spans="2:8" ht="18.75" customHeight="1">
       <c r="B77" s="1"/>
-      <c r="C77" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="D77" s="63">
-        <v>345</v>
-      </c>
-      <c r="E77" s="65">
-        <v>82213</v>
+      <c r="C77" s="60"/>
+      <c r="D77" s="61">
+        <v>187</v>
+      </c>
+      <c r="E77" s="64">
+        <v>5365</v>
       </c>
       <c r="F77" s="33"/>
       <c r="G77" s="2"/>
@@ -2271,14 +2269,14 @@
     </row>
     <row r="78" spans="2:8" ht="18.75" customHeight="1">
       <c r="B78" s="1"/>
-      <c r="C78" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="D78" s="42">
-        <v>346</v>
-      </c>
-      <c r="E78" s="43">
-        <v>76220</v>
+      <c r="C78" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="D78" s="63">
+        <v>345</v>
+      </c>
+      <c r="E78" s="65">
+        <v>82213</v>
       </c>
       <c r="F78" s="33"/>
       <c r="G78" s="2"/>
@@ -2286,12 +2284,14 @@
     </row>
     <row r="79" spans="2:8" ht="18.75" customHeight="1">
       <c r="B79" s="1"/>
-      <c r="C79" s="41"/>
+      <c r="C79" s="41" t="s">
+        <v>31</v>
+      </c>
       <c r="D79" s="42">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E79" s="43">
-        <v>73576</v>
+        <v>76220</v>
       </c>
       <c r="F79" s="33"/>
       <c r="G79" s="2"/>
@@ -2301,10 +2301,10 @@
       <c r="B80" s="1"/>
       <c r="C80" s="41"/>
       <c r="D80" s="42">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="E80" s="43">
-        <v>70842</v>
+        <v>73576</v>
       </c>
       <c r="F80" s="33"/>
       <c r="G80" s="2"/>
@@ -2314,10 +2314,10 @@
       <c r="B81" s="1"/>
       <c r="C81" s="41"/>
       <c r="D81" s="42">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="E81" s="43">
-        <v>69857</v>
+        <v>70842</v>
       </c>
       <c r="F81" s="33"/>
       <c r="G81" s="2"/>
@@ -2327,10 +2327,10 @@
       <c r="B82" s="1"/>
       <c r="C82" s="41"/>
       <c r="D82" s="42">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="E82" s="43">
-        <v>90202</v>
+        <v>69857</v>
       </c>
       <c r="F82" s="33"/>
       <c r="G82" s="2"/>
@@ -2340,10 +2340,10 @@
       <c r="B83" s="1"/>
       <c r="C83" s="41"/>
       <c r="D83" s="42">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="E83" s="43">
-        <v>72115</v>
+        <v>90202</v>
       </c>
       <c r="F83" s="33"/>
       <c r="G83" s="2"/>
@@ -2353,10 +2353,10 @@
       <c r="B84" s="1"/>
       <c r="C84" s="41"/>
       <c r="D84" s="42">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E84" s="43">
-        <v>69178</v>
+        <v>72115</v>
       </c>
       <c r="F84" s="33"/>
       <c r="G84" s="2"/>
@@ -2366,10 +2366,10 @@
       <c r="B85" s="1"/>
       <c r="C85" s="41"/>
       <c r="D85" s="42">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E85" s="43">
-        <v>68020</v>
+        <v>69178</v>
       </c>
       <c r="F85" s="33"/>
       <c r="G85" s="2"/>
@@ -2379,10 +2379,10 @@
       <c r="B86" s="1"/>
       <c r="C86" s="41"/>
       <c r="D86" s="42">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="E86" s="43">
-        <v>62719</v>
+        <v>68020</v>
       </c>
       <c r="F86" s="33"/>
       <c r="G86" s="2"/>
@@ -2392,10 +2392,10 @@
       <c r="B87" s="1"/>
       <c r="C87" s="41"/>
       <c r="D87" s="42">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E87" s="43">
-        <v>62896</v>
+        <v>62719</v>
       </c>
       <c r="F87" s="33"/>
       <c r="G87" s="2"/>
@@ -2405,10 +2405,10 @@
       <c r="B88" s="1"/>
       <c r="C88" s="41"/>
       <c r="D88" s="42">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E88" s="43">
-        <v>66567</v>
+        <v>62896</v>
       </c>
       <c r="F88" s="33"/>
       <c r="G88" s="2"/>
@@ -2418,10 +2418,10 @@
       <c r="B89" s="1"/>
       <c r="C89" s="41"/>
       <c r="D89" s="42">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E89" s="43">
-        <v>66923</v>
+        <v>66567</v>
       </c>
       <c r="F89" s="33"/>
       <c r="G89" s="2"/>
@@ -2431,10 +2431,10 @@
       <c r="B90" s="1"/>
       <c r="C90" s="41"/>
       <c r="D90" s="42">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="E90" s="43">
-        <v>59112</v>
+        <v>66923</v>
       </c>
       <c r="F90" s="33"/>
       <c r="G90" s="2"/>
@@ -2444,10 +2444,10 @@
       <c r="B91" s="1"/>
       <c r="C91" s="41"/>
       <c r="D91" s="42">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="E91" s="43">
-        <v>74337</v>
+        <v>59112</v>
       </c>
       <c r="F91" s="33"/>
       <c r="G91" s="2"/>
@@ -2457,10 +2457,10 @@
       <c r="B92" s="1"/>
       <c r="C92" s="41"/>
       <c r="D92" s="42">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="E92" s="43">
-        <v>74814</v>
+        <v>74337</v>
       </c>
       <c r="F92" s="33"/>
       <c r="G92" s="2"/>
@@ -2470,10 +2470,10 @@
       <c r="B93" s="1"/>
       <c r="C93" s="41"/>
       <c r="D93" s="42">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E93" s="43">
-        <v>72826</v>
+        <v>74814</v>
       </c>
       <c r="F93" s="33"/>
       <c r="G93" s="2"/>
@@ -2483,10 +2483,10 @@
       <c r="B94" s="1"/>
       <c r="C94" s="41"/>
       <c r="D94" s="42">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="E94" s="43">
-        <v>68659</v>
+        <v>72826</v>
       </c>
       <c r="F94" s="33"/>
       <c r="G94" s="2"/>
@@ -2496,10 +2496,10 @@
       <c r="B95" s="1"/>
       <c r="C95" s="41"/>
       <c r="D95" s="42">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="E95" s="43">
-        <v>67081</v>
+        <v>68659</v>
       </c>
       <c r="F95" s="33"/>
       <c r="G95" s="2"/>
@@ -2509,10 +2509,10 @@
       <c r="B96" s="1"/>
       <c r="C96" s="41"/>
       <c r="D96" s="42">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E96" s="43">
-        <v>68985</v>
+        <v>67081</v>
       </c>
       <c r="F96" s="33"/>
       <c r="G96" s="2"/>
@@ -2522,10 +2522,10 @@
       <c r="B97" s="1"/>
       <c r="C97" s="41"/>
       <c r="D97" s="42">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="E97" s="43">
-        <v>70339</v>
+        <v>68985</v>
       </c>
       <c r="F97" s="33"/>
       <c r="G97" s="2"/>
@@ -2535,10 +2535,10 @@
       <c r="B98" s="1"/>
       <c r="C98" s="41"/>
       <c r="D98" s="42">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="E98" s="43">
-        <v>74868</v>
+        <v>70339</v>
       </c>
       <c r="F98" s="33"/>
       <c r="G98" s="2"/>
@@ -2548,10 +2548,10 @@
       <c r="B99" s="1"/>
       <c r="C99" s="41"/>
       <c r="D99" s="42">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="E99" s="43">
-        <v>69628</v>
+        <v>74868</v>
       </c>
       <c r="F99" s="33"/>
       <c r="G99" s="2"/>
@@ -2561,10 +2561,10 @@
       <c r="B100" s="1"/>
       <c r="C100" s="41"/>
       <c r="D100" s="42">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="E100" s="43">
-        <v>74336</v>
+        <v>69628</v>
       </c>
       <c r="F100" s="33"/>
       <c r="G100" s="2"/>
@@ -2574,10 +2574,10 @@
       <c r="B101" s="1"/>
       <c r="C101" s="41"/>
       <c r="D101" s="42">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E101" s="43">
-        <v>69325</v>
+        <v>74336</v>
       </c>
       <c r="F101" s="33"/>
       <c r="G101" s="2"/>
@@ -2587,10 +2587,10 @@
       <c r="B102" s="1"/>
       <c r="C102" s="41"/>
       <c r="D102" s="42">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E102" s="43">
-        <v>68143</v>
+        <v>69325</v>
       </c>
       <c r="F102" s="33"/>
       <c r="G102" s="2"/>
@@ -2600,10 +2600,10 @@
       <c r="B103" s="1"/>
       <c r="C103" s="41"/>
       <c r="D103" s="42">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E103" s="43">
-        <v>62854</v>
+        <v>68143</v>
       </c>
       <c r="F103" s="33"/>
       <c r="G103" s="2"/>
@@ -2613,10 +2613,10 @@
       <c r="B104" s="1"/>
       <c r="C104" s="41"/>
       <c r="D104" s="42">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E104" s="43">
-        <v>57769</v>
+        <v>62854</v>
       </c>
       <c r="F104" s="33"/>
       <c r="G104" s="2"/>
@@ -2626,10 +2626,10 @@
       <c r="B105" s="1"/>
       <c r="C105" s="41"/>
       <c r="D105" s="42">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E105" s="43">
-        <v>42282</v>
+        <v>57769</v>
       </c>
       <c r="F105" s="33"/>
       <c r="G105" s="2"/>
@@ -2639,10 +2639,10 @@
       <c r="B106" s="1"/>
       <c r="C106" s="41"/>
       <c r="D106" s="42">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E106" s="43">
-        <v>38562</v>
+        <v>42282</v>
       </c>
       <c r="F106" s="33"/>
       <c r="G106" s="2"/>
@@ -2652,10 +2652,10 @@
       <c r="B107" s="1"/>
       <c r="C107" s="41"/>
       <c r="D107" s="42">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E107" s="43">
-        <v>36707</v>
+        <v>38562</v>
       </c>
       <c r="F107" s="33"/>
       <c r="G107" s="2"/>
@@ -2665,10 +2665,10 @@
       <c r="B108" s="1"/>
       <c r="C108" s="41"/>
       <c r="D108" s="42">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E108" s="43">
-        <v>25699</v>
+        <v>36707</v>
       </c>
       <c r="F108" s="33"/>
       <c r="G108" s="2"/>
@@ -2678,10 +2678,10 @@
       <c r="B109" s="1"/>
       <c r="C109" s="41"/>
       <c r="D109" s="42">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="E109" s="43">
-        <v>26558</v>
+        <v>25699</v>
       </c>
       <c r="F109" s="33"/>
       <c r="G109" s="2"/>
@@ -2691,10 +2691,10 @@
       <c r="B110" s="1"/>
       <c r="C110" s="41"/>
       <c r="D110" s="42">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E110" s="43">
-        <v>23311</v>
+        <v>26558</v>
       </c>
       <c r="F110" s="33"/>
       <c r="G110" s="2"/>
@@ -2704,10 +2704,10 @@
       <c r="B111" s="1"/>
       <c r="C111" s="41"/>
       <c r="D111" s="42">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E111" s="43">
-        <v>13512</v>
+        <v>23311</v>
       </c>
       <c r="F111" s="33"/>
       <c r="G111" s="2"/>
@@ -2717,10 +2717,10 @@
       <c r="B112" s="1"/>
       <c r="C112" s="41"/>
       <c r="D112" s="42">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E112" s="43">
-        <v>5131</v>
+        <v>13512</v>
       </c>
       <c r="F112" s="33"/>
       <c r="G112" s="2"/>
@@ -2730,10 +2730,10 @@
       <c r="B113" s="1"/>
       <c r="C113" s="41"/>
       <c r="D113" s="42">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="E113" s="43">
-        <v>7221</v>
+        <v>5131</v>
       </c>
       <c r="F113" s="33"/>
       <c r="G113" s="2"/>
@@ -2743,10 +2743,10 @@
       <c r="B114" s="1"/>
       <c r="C114" s="41"/>
       <c r="D114" s="42">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="E114" s="43">
-        <v>6852</v>
+        <v>7221</v>
       </c>
       <c r="F114" s="33"/>
       <c r="G114" s="2"/>
@@ -2754,12 +2754,12 @@
     </row>
     <row r="115" spans="2:8" ht="18.75" customHeight="1">
       <c r="B115" s="1"/>
-      <c r="C115" s="60"/>
-      <c r="D115" s="61">
-        <v>383</v>
-      </c>
-      <c r="E115" s="64">
-        <v>4741</v>
+      <c r="C115" s="41"/>
+      <c r="D115" s="42">
+        <v>382</v>
+      </c>
+      <c r="E115" s="43">
+        <v>6852</v>
       </c>
       <c r="F115" s="33"/>
       <c r="G115" s="2"/>
@@ -2767,14 +2767,12 @@
     </row>
     <row r="116" spans="2:8" ht="18.75" customHeight="1">
       <c r="B116" s="1"/>
-      <c r="C116" s="62" t="s">
-        <v>21</v>
-      </c>
-      <c r="D116" s="63">
-        <v>92</v>
-      </c>
-      <c r="E116" s="65">
-        <v>17984</v>
+      <c r="C116" s="60"/>
+      <c r="D116" s="61">
+        <v>383</v>
+      </c>
+      <c r="E116" s="64">
+        <v>4741</v>
       </c>
       <c r="F116" s="33"/>
       <c r="G116" s="2"/>
@@ -2782,14 +2780,14 @@
     </row>
     <row r="117" spans="2:8" ht="18.75" customHeight="1">
       <c r="B117" s="1"/>
-      <c r="C117" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="D117" s="42">
-        <v>93</v>
-      </c>
-      <c r="E117" s="43">
-        <v>8346</v>
+      <c r="C117" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="D117" s="63">
+        <v>92</v>
+      </c>
+      <c r="E117" s="65">
+        <v>18104</v>
       </c>
       <c r="F117" s="33"/>
       <c r="G117" s="2"/>
@@ -2797,12 +2795,14 @@
     </row>
     <row r="118" spans="2:8" ht="18.75" customHeight="1">
       <c r="B118" s="1"/>
-      <c r="C118" s="41"/>
+      <c r="C118" s="41" t="s">
+        <v>32</v>
+      </c>
       <c r="D118" s="42">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E118" s="43">
-        <v>10783</v>
+        <v>8346</v>
       </c>
       <c r="F118" s="33"/>
       <c r="G118" s="2"/>
@@ -2812,10 +2812,10 @@
       <c r="B119" s="1"/>
       <c r="C119" s="41"/>
       <c r="D119" s="42">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E119" s="43">
-        <v>15820</v>
+        <v>10783</v>
       </c>
       <c r="F119" s="33"/>
       <c r="G119" s="2"/>
@@ -2825,10 +2825,10 @@
       <c r="B120" s="1"/>
       <c r="C120" s="41"/>
       <c r="D120" s="42">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E120" s="43">
-        <v>7089</v>
+        <v>15820</v>
       </c>
       <c r="F120" s="33"/>
       <c r="G120" s="2"/>
@@ -2838,10 +2838,10 @@
       <c r="B121" s="1"/>
       <c r="C121" s="41"/>
       <c r="D121" s="42">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E121" s="43">
-        <v>11311</v>
+        <v>7089</v>
       </c>
       <c r="F121" s="33"/>
       <c r="G121" s="2"/>
@@ -2851,10 +2851,10 @@
       <c r="B122" s="1"/>
       <c r="C122" s="41"/>
       <c r="D122" s="42">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E122" s="43">
-        <v>6695</v>
+        <v>11311</v>
       </c>
       <c r="F122" s="33"/>
       <c r="G122" s="2"/>
@@ -2864,10 +2864,10 @@
       <c r="B123" s="1"/>
       <c r="C123" s="41"/>
       <c r="D123" s="42">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E123" s="43">
-        <v>14138</v>
+        <v>6711</v>
       </c>
       <c r="F123" s="33"/>
       <c r="G123" s="2"/>
@@ -2877,10 +2877,10 @@
       <c r="B124" s="1"/>
       <c r="C124" s="41"/>
       <c r="D124" s="42">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E124" s="43">
-        <v>6481</v>
+        <v>14138</v>
       </c>
       <c r="F124" s="33"/>
       <c r="G124" s="2"/>
@@ -2890,10 +2890,10 @@
       <c r="B125" s="1"/>
       <c r="C125" s="41"/>
       <c r="D125" s="42">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E125" s="43">
-        <v>4969</v>
+        <v>6481</v>
       </c>
       <c r="F125" s="33"/>
       <c r="G125" s="2"/>
@@ -2903,10 +2903,10 @@
       <c r="B126" s="1"/>
       <c r="C126" s="41"/>
       <c r="D126" s="42">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E126" s="43">
-        <v>4283</v>
+        <v>4969</v>
       </c>
       <c r="F126" s="33"/>
       <c r="G126" s="2"/>
@@ -2916,10 +2916,10 @@
       <c r="B127" s="1"/>
       <c r="C127" s="41"/>
       <c r="D127" s="42">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E127" s="43">
-        <v>5777</v>
+        <v>4283</v>
       </c>
       <c r="F127" s="33"/>
       <c r="G127" s="2"/>
@@ -2929,10 +2929,10 @@
       <c r="B128" s="1"/>
       <c r="C128" s="41"/>
       <c r="D128" s="42">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E128" s="43">
-        <v>4159</v>
+        <v>5777</v>
       </c>
       <c r="F128" s="33"/>
       <c r="G128" s="2"/>
@@ -2942,10 +2942,10 @@
       <c r="B129" s="1"/>
       <c r="C129" s="41"/>
       <c r="D129" s="42">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E129" s="43">
-        <v>10394</v>
+        <v>4159</v>
       </c>
       <c r="F129" s="33"/>
       <c r="G129" s="2"/>
@@ -2955,10 +2955,10 @@
       <c r="B130" s="1"/>
       <c r="C130" s="41"/>
       <c r="D130" s="42">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E130" s="43">
-        <v>5297</v>
+        <v>10394</v>
       </c>
       <c r="F130" s="33"/>
       <c r="G130" s="2"/>
@@ -2968,10 +2968,10 @@
       <c r="B131" s="1"/>
       <c r="C131" s="41"/>
       <c r="D131" s="42">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E131" s="43">
-        <v>9359</v>
+        <v>5388</v>
       </c>
       <c r="F131" s="33"/>
       <c r="G131" s="2"/>
@@ -2981,10 +2981,10 @@
       <c r="B132" s="1"/>
       <c r="C132" s="41"/>
       <c r="D132" s="42">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E132" s="43">
-        <v>15938</v>
+        <v>9359</v>
       </c>
       <c r="F132" s="33"/>
       <c r="G132" s="2"/>
@@ -2994,10 +2994,10 @@
       <c r="B133" s="1"/>
       <c r="C133" s="41"/>
       <c r="D133" s="42">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E133" s="43">
-        <v>7189</v>
+        <v>15938</v>
       </c>
       <c r="F133" s="33"/>
       <c r="G133" s="2"/>
@@ -3007,10 +3007,10 @@
       <c r="B134" s="1"/>
       <c r="C134" s="41"/>
       <c r="D134" s="42">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E134" s="43">
-        <v>8143</v>
+        <v>7189</v>
       </c>
       <c r="F134" s="33"/>
       <c r="G134" s="2"/>
@@ -3020,10 +3020,10 @@
       <c r="B135" s="1"/>
       <c r="C135" s="41"/>
       <c r="D135" s="42">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E135" s="43">
-        <v>7010</v>
+        <v>8143</v>
       </c>
       <c r="F135" s="33"/>
       <c r="G135" s="2"/>
@@ -3033,10 +3033,10 @@
       <c r="B136" s="1"/>
       <c r="C136" s="41"/>
       <c r="D136" s="42">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E136" s="43">
-        <v>11873</v>
+        <v>7090</v>
       </c>
       <c r="F136" s="33"/>
       <c r="G136" s="2"/>
@@ -3046,10 +3046,10 @@
       <c r="B137" s="1"/>
       <c r="C137" s="41"/>
       <c r="D137" s="42">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E137" s="43">
-        <v>32420</v>
+        <v>11895</v>
       </c>
       <c r="F137" s="33"/>
       <c r="G137" s="2"/>
@@ -3059,10 +3059,10 @@
       <c r="B138" s="1"/>
       <c r="C138" s="41"/>
       <c r="D138" s="42">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E138" s="43">
-        <v>18802</v>
+        <v>32420</v>
       </c>
       <c r="F138" s="33"/>
       <c r="G138" s="2"/>
@@ -3072,10 +3072,10 @@
       <c r="B139" s="1"/>
       <c r="C139" s="41"/>
       <c r="D139" s="42">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E139" s="43">
-        <v>7764</v>
+        <v>18802</v>
       </c>
       <c r="F139" s="33"/>
       <c r="G139" s="2"/>
@@ -3085,10 +3085,10 @@
       <c r="B140" s="1"/>
       <c r="C140" s="41"/>
       <c r="D140" s="42">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E140" s="43">
-        <v>11288</v>
+        <v>7764</v>
       </c>
       <c r="F140" s="33"/>
       <c r="G140" s="2"/>
@@ -3098,10 +3098,10 @@
       <c r="B141" s="1"/>
       <c r="C141" s="41"/>
       <c r="D141" s="42">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E141" s="43">
-        <v>21846</v>
+        <v>11288</v>
       </c>
       <c r="F141" s="33"/>
       <c r="G141" s="2"/>
@@ -3111,10 +3111,10 @@
       <c r="B142" s="1"/>
       <c r="C142" s="41"/>
       <c r="D142" s="42">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E142" s="43">
-        <v>8858</v>
+        <v>21846</v>
       </c>
       <c r="F142" s="33"/>
       <c r="G142" s="2"/>
@@ -3124,10 +3124,10 @@
       <c r="B143" s="1"/>
       <c r="C143" s="41"/>
       <c r="D143" s="42">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E143" s="43">
-        <v>8845</v>
+        <v>8858</v>
       </c>
       <c r="F143" s="33"/>
       <c r="G143" s="2"/>
@@ -3137,10 +3137,10 @@
       <c r="B144" s="1"/>
       <c r="C144" s="41"/>
       <c r="D144" s="42">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E144" s="43">
-        <v>11288</v>
+        <v>8845</v>
       </c>
       <c r="F144" s="33"/>
       <c r="G144" s="2"/>
@@ -3150,10 +3150,10 @@
       <c r="B145" s="1"/>
       <c r="C145" s="41"/>
       <c r="D145" s="42">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E145" s="43">
-        <v>18363</v>
+        <v>11288</v>
       </c>
       <c r="F145" s="33"/>
       <c r="G145" s="2"/>
@@ -3163,10 +3163,10 @@
       <c r="B146" s="1"/>
       <c r="C146" s="41"/>
       <c r="D146" s="42">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E146" s="43">
-        <v>11178</v>
+        <v>18363</v>
       </c>
       <c r="F146" s="33"/>
       <c r="G146" s="2"/>
@@ -3176,10 +3176,10 @@
       <c r="B147" s="1"/>
       <c r="C147" s="41"/>
       <c r="D147" s="42">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E147" s="43">
-        <v>13604</v>
+        <v>11178</v>
       </c>
       <c r="F147" s="33"/>
       <c r="G147" s="2"/>
@@ -3189,10 +3189,10 @@
       <c r="B148" s="1"/>
       <c r="C148" s="41"/>
       <c r="D148" s="42">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E148" s="43">
-        <v>10402</v>
+        <v>13604</v>
       </c>
       <c r="F148" s="33"/>
       <c r="G148" s="2"/>
@@ -3202,10 +3202,10 @@
       <c r="B149" s="1"/>
       <c r="C149" s="41"/>
       <c r="D149" s="42">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E149" s="43">
-        <v>8101</v>
+        <v>10402</v>
       </c>
       <c r="F149" s="33"/>
       <c r="G149" s="2"/>
@@ -3215,10 +3215,10 @@
       <c r="B150" s="1"/>
       <c r="C150" s="41"/>
       <c r="D150" s="42">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E150" s="43">
-        <v>6808</v>
+        <v>8101</v>
       </c>
       <c r="F150" s="33"/>
       <c r="G150" s="2"/>
@@ -3228,10 +3228,10 @@
       <c r="B151" s="1"/>
       <c r="C151" s="41"/>
       <c r="D151" s="42">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E151" s="43">
-        <v>8463</v>
+        <v>6808</v>
       </c>
       <c r="F151" s="33"/>
       <c r="G151" s="2"/>
@@ -3241,10 +3241,10 @@
       <c r="B152" s="1"/>
       <c r="C152" s="41"/>
       <c r="D152" s="42">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E152" s="43">
-        <v>17194</v>
+        <v>8463</v>
       </c>
       <c r="F152" s="33"/>
       <c r="G152" s="2"/>
@@ -3254,10 +3254,10 @@
       <c r="B153" s="1"/>
       <c r="C153" s="41"/>
       <c r="D153" s="42">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E153" s="43">
-        <v>10301</v>
+        <v>17194</v>
       </c>
       <c r="F153" s="33"/>
       <c r="G153" s="2"/>
@@ -3267,10 +3267,10 @@
       <c r="B154" s="1"/>
       <c r="C154" s="41"/>
       <c r="D154" s="42">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E154" s="43">
-        <v>12732</v>
+        <v>10301</v>
       </c>
       <c r="F154" s="33"/>
       <c r="G154" s="2"/>
@@ -3280,10 +3280,10 @@
       <c r="B155" s="1"/>
       <c r="C155" s="41"/>
       <c r="D155" s="42">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E155" s="43">
-        <v>8001</v>
+        <v>12732</v>
       </c>
       <c r="F155" s="33"/>
       <c r="G155" s="2"/>
@@ -3293,10 +3293,10 @@
       <c r="B156" s="1"/>
       <c r="C156" s="41"/>
       <c r="D156" s="42">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E156" s="43">
-        <v>9517</v>
+        <v>8001</v>
       </c>
       <c r="F156" s="33"/>
       <c r="G156" s="2"/>
@@ -3306,10 +3306,10 @@
       <c r="B157" s="1"/>
       <c r="C157" s="41"/>
       <c r="D157" s="42">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E157" s="43">
-        <v>9999</v>
+        <v>9517</v>
       </c>
       <c r="F157" s="33"/>
       <c r="G157" s="2"/>
@@ -3319,10 +3319,10 @@
       <c r="B158" s="1"/>
       <c r="C158" s="41"/>
       <c r="D158" s="42">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E158" s="43">
-        <v>7737</v>
+        <v>9999</v>
       </c>
       <c r="F158" s="33"/>
       <c r="G158" s="2"/>
@@ -3332,10 +3332,10 @@
       <c r="B159" s="1"/>
       <c r="C159" s="41"/>
       <c r="D159" s="42">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E159" s="43">
-        <v>7260</v>
+        <v>7737</v>
       </c>
       <c r="F159" s="33"/>
       <c r="G159" s="2"/>
@@ -3345,10 +3345,10 @@
       <c r="B160" s="1"/>
       <c r="C160" s="41"/>
       <c r="D160" s="42">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E160" s="43">
-        <v>8132</v>
+        <v>7260</v>
       </c>
       <c r="F160" s="33"/>
       <c r="G160" s="2"/>
@@ -3358,10 +3358,10 @@
       <c r="B161" s="1"/>
       <c r="C161" s="41"/>
       <c r="D161" s="42">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E161" s="43">
-        <v>8896</v>
+        <v>8132</v>
       </c>
       <c r="F161" s="33"/>
       <c r="G161" s="2"/>
@@ -3371,10 +3371,10 @@
       <c r="B162" s="1"/>
       <c r="C162" s="41"/>
       <c r="D162" s="42">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E162" s="43">
-        <v>10869</v>
+        <v>8896</v>
       </c>
       <c r="F162" s="33"/>
       <c r="G162" s="2"/>
@@ -3384,10 +3384,10 @@
       <c r="B163" s="1"/>
       <c r="C163" s="41"/>
       <c r="D163" s="42">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E163" s="43">
-        <v>11361</v>
+        <v>10869</v>
       </c>
       <c r="F163" s="33"/>
       <c r="G163" s="2"/>
@@ -3397,10 +3397,10 @@
       <c r="B164" s="1"/>
       <c r="C164" s="41"/>
       <c r="D164" s="42">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E164" s="43">
-        <v>24319</v>
+        <v>11361</v>
       </c>
       <c r="F164" s="33"/>
       <c r="G164" s="2"/>
@@ -3410,10 +3410,10 @@
       <c r="B165" s="1"/>
       <c r="C165" s="41"/>
       <c r="D165" s="42">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E165" s="43">
-        <v>14711</v>
+        <v>24319</v>
       </c>
       <c r="F165" s="33"/>
       <c r="G165" s="2"/>
@@ -3423,10 +3423,10 @@
       <c r="B166" s="1"/>
       <c r="C166" s="41"/>
       <c r="D166" s="42">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E166" s="43">
-        <v>11623</v>
+        <v>14711</v>
       </c>
       <c r="F166" s="33"/>
       <c r="G166" s="2"/>
@@ -3436,10 +3436,10 @@
       <c r="B167" s="1"/>
       <c r="C167" s="41"/>
       <c r="D167" s="42">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E167" s="43">
-        <v>19984</v>
+        <v>11623</v>
       </c>
       <c r="F167" s="33"/>
       <c r="G167" s="2"/>
@@ -3449,10 +3449,10 @@
       <c r="B168" s="1"/>
       <c r="C168" s="41"/>
       <c r="D168" s="42">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E168" s="43">
-        <v>12792</v>
+        <v>19984</v>
       </c>
       <c r="F168" s="33"/>
       <c r="G168" s="2"/>
@@ -3462,10 +3462,10 @@
       <c r="B169" s="1"/>
       <c r="C169" s="41"/>
       <c r="D169" s="42">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E169" s="43">
-        <v>30462</v>
+        <v>12792</v>
       </c>
       <c r="F169" s="33"/>
       <c r="G169" s="2"/>
@@ -3475,10 +3475,10 @@
       <c r="B170" s="1"/>
       <c r="C170" s="41"/>
       <c r="D170" s="42">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E170" s="43">
-        <v>30077</v>
+        <v>30462</v>
       </c>
       <c r="F170" s="33"/>
       <c r="G170" s="2"/>
@@ -3488,10 +3488,10 @@
       <c r="B171" s="1"/>
       <c r="C171" s="41"/>
       <c r="D171" s="42">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E171" s="43">
-        <v>33982</v>
+        <v>30077</v>
       </c>
       <c r="F171" s="33"/>
       <c r="G171" s="2"/>
@@ -3501,10 +3501,10 @@
       <c r="B172" s="1"/>
       <c r="C172" s="41"/>
       <c r="D172" s="42">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E172" s="43">
-        <v>24786</v>
+        <v>33982</v>
       </c>
       <c r="F172" s="33"/>
       <c r="G172" s="2"/>
@@ -3514,10 +3514,10 @@
       <c r="B173" s="1"/>
       <c r="C173" s="41"/>
       <c r="D173" s="42">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E173" s="43">
-        <v>26668</v>
+        <v>24786</v>
       </c>
       <c r="F173" s="33"/>
       <c r="G173" s="2"/>
@@ -3527,10 +3527,10 @@
       <c r="B174" s="1"/>
       <c r="C174" s="41"/>
       <c r="D174" s="42">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E174" s="43">
-        <v>26644</v>
+        <v>26668</v>
       </c>
       <c r="F174" s="33"/>
       <c r="G174" s="2"/>
@@ -3540,10 +3540,10 @@
       <c r="B175" s="1"/>
       <c r="C175" s="41"/>
       <c r="D175" s="42">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E175" s="43">
-        <v>28063</v>
+        <v>26644</v>
       </c>
       <c r="F175" s="33"/>
       <c r="G175" s="2"/>
@@ -3553,10 +3553,10 @@
       <c r="B176" s="1"/>
       <c r="C176" s="41"/>
       <c r="D176" s="42">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E176" s="43">
-        <v>23110</v>
+        <v>28063</v>
       </c>
       <c r="F176" s="33"/>
       <c r="G176" s="2"/>
@@ -3566,10 +3566,10 @@
       <c r="B177" s="1"/>
       <c r="C177" s="41"/>
       <c r="D177" s="42">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E177" s="43">
-        <v>28546</v>
+        <v>23110</v>
       </c>
       <c r="F177" s="33"/>
       <c r="G177" s="2"/>
@@ -3579,10 +3579,10 @@
       <c r="B178" s="1"/>
       <c r="C178" s="41"/>
       <c r="D178" s="42">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E178" s="43">
-        <v>24396</v>
+        <v>28546</v>
       </c>
       <c r="F178" s="33"/>
       <c r="G178" s="2"/>
@@ -3592,10 +3592,10 @@
       <c r="B179" s="1"/>
       <c r="C179" s="41"/>
       <c r="D179" s="42">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E179" s="43">
-        <v>23472</v>
+        <v>24396</v>
       </c>
       <c r="F179" s="33"/>
       <c r="G179" s="2"/>
@@ -3605,10 +3605,10 @@
       <c r="B180" s="1"/>
       <c r="C180" s="41"/>
       <c r="D180" s="42">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E180" s="43">
-        <v>24011</v>
+        <v>23472</v>
       </c>
       <c r="F180" s="33"/>
       <c r="G180" s="2"/>
@@ -3618,10 +3618,10 @@
       <c r="B181" s="1"/>
       <c r="C181" s="41"/>
       <c r="D181" s="42">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E181" s="43">
-        <v>26163</v>
+        <v>24011</v>
       </c>
       <c r="F181" s="33"/>
       <c r="G181" s="2"/>
@@ -3631,10 +3631,10 @@
       <c r="B182" s="1"/>
       <c r="C182" s="41"/>
       <c r="D182" s="42">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E182" s="43">
-        <v>25894</v>
+        <v>26163</v>
       </c>
       <c r="F182" s="33"/>
       <c r="G182" s="2"/>
@@ -3644,10 +3644,10 @@
       <c r="B183" s="1"/>
       <c r="C183" s="41"/>
       <c r="D183" s="42">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E183" s="43">
-        <v>18790</v>
+        <v>25894</v>
       </c>
       <c r="F183" s="33"/>
       <c r="G183" s="2"/>
@@ -3657,10 +3657,10 @@
       <c r="B184" s="1"/>
       <c r="C184" s="41"/>
       <c r="D184" s="42">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E184" s="43">
-        <v>16740</v>
+        <v>18790</v>
       </c>
       <c r="F184" s="33"/>
       <c r="G184" s="2"/>
@@ -3670,10 +3670,10 @@
       <c r="B185" s="1"/>
       <c r="C185" s="41"/>
       <c r="D185" s="42">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E185" s="43">
-        <v>19557</v>
+        <v>16752</v>
       </c>
       <c r="F185" s="33"/>
       <c r="G185" s="2"/>
@@ -3683,10 +3683,10 @@
       <c r="B186" s="1"/>
       <c r="C186" s="41"/>
       <c r="D186" s="42">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E186" s="43">
-        <v>14769</v>
+        <v>19557</v>
       </c>
       <c r="F186" s="33"/>
       <c r="G186" s="2"/>
@@ -3696,10 +3696,10 @@
       <c r="B187" s="1"/>
       <c r="C187" s="41"/>
       <c r="D187" s="42">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E187" s="43">
-        <v>18285</v>
+        <v>14780</v>
       </c>
       <c r="F187" s="33"/>
       <c r="G187" s="2"/>
@@ -3709,10 +3709,10 @@
       <c r="B188" s="1"/>
       <c r="C188" s="41"/>
       <c r="D188" s="42">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E188" s="43">
-        <v>23415</v>
+        <v>18285</v>
       </c>
       <c r="F188" s="33"/>
       <c r="G188" s="2"/>
@@ -3722,10 +3722,10 @@
       <c r="B189" s="1"/>
       <c r="C189" s="41"/>
       <c r="D189" s="42">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E189" s="43">
-        <v>11203</v>
+        <v>23689</v>
       </c>
       <c r="F189" s="33"/>
       <c r="G189" s="2"/>
@@ -3735,10 +3735,10 @@
       <c r="B190" s="1"/>
       <c r="C190" s="41"/>
       <c r="D190" s="42">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E190" s="43">
-        <v>12813</v>
+        <v>11249</v>
       </c>
       <c r="F190" s="33"/>
       <c r="G190" s="2"/>
@@ -3748,10 +3748,10 @@
       <c r="B191" s="1"/>
       <c r="C191" s="41"/>
       <c r="D191" s="42">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E191" s="43">
-        <v>13835</v>
+        <v>12813</v>
       </c>
       <c r="F191" s="33"/>
       <c r="G191" s="2"/>
@@ -3761,10 +3761,10 @@
       <c r="B192" s="1"/>
       <c r="C192" s="41"/>
       <c r="D192" s="42">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E192" s="43">
-        <v>11153</v>
+        <v>13885</v>
       </c>
       <c r="F192" s="33"/>
       <c r="G192" s="2"/>
@@ -3774,10 +3774,10 @@
       <c r="B193" s="1"/>
       <c r="C193" s="41"/>
       <c r="D193" s="42">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E193" s="43">
-        <v>11019</v>
+        <v>11153</v>
       </c>
       <c r="F193" s="33"/>
       <c r="G193" s="2"/>
@@ -3787,10 +3787,10 @@
       <c r="B194" s="1"/>
       <c r="C194" s="41"/>
       <c r="D194" s="42">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E194" s="43">
-        <v>8643</v>
+        <v>11019</v>
       </c>
       <c r="F194" s="33"/>
       <c r="G194" s="2"/>
@@ -3800,10 +3800,10 @@
       <c r="B195" s="1"/>
       <c r="C195" s="41"/>
       <c r="D195" s="42">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E195" s="43">
-        <v>3144</v>
+        <v>8643</v>
       </c>
       <c r="F195" s="33"/>
       <c r="G195" s="2"/>
@@ -3813,10 +3813,10 @@
       <c r="B196" s="1"/>
       <c r="C196" s="41"/>
       <c r="D196" s="42">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E196" s="43">
-        <v>2925</v>
+        <v>3144</v>
       </c>
       <c r="F196" s="33"/>
       <c r="G196" s="2"/>
@@ -3826,10 +3826,10 @@
       <c r="B197" s="1"/>
       <c r="C197" s="41"/>
       <c r="D197" s="42">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E197" s="43">
-        <v>6107</v>
+        <v>2925</v>
       </c>
       <c r="F197" s="33"/>
       <c r="G197" s="2"/>
@@ -3839,10 +3839,10 @@
       <c r="B198" s="1"/>
       <c r="C198" s="41"/>
       <c r="D198" s="42">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E198" s="43">
-        <v>4706</v>
+        <v>6107</v>
       </c>
       <c r="F198" s="33"/>
       <c r="G198" s="2"/>
@@ -3852,10 +3852,10 @@
       <c r="B199" s="1"/>
       <c r="C199" s="41"/>
       <c r="D199" s="42">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E199" s="43">
-        <v>4716</v>
+        <v>4706</v>
       </c>
       <c r="F199" s="33"/>
       <c r="G199" s="2"/>
@@ -3865,10 +3865,10 @@
       <c r="B200" s="1"/>
       <c r="C200" s="41"/>
       <c r="D200" s="42">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E200" s="43">
-        <v>7743</v>
+        <v>4716</v>
       </c>
       <c r="F200" s="33"/>
       <c r="G200" s="2"/>
@@ -3878,10 +3878,10 @@
       <c r="B201" s="1"/>
       <c r="C201" s="41"/>
       <c r="D201" s="42">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E201" s="43">
-        <v>5284</v>
+        <v>7743</v>
       </c>
       <c r="F201" s="33"/>
       <c r="G201" s="2"/>
@@ -3891,10 +3891,10 @@
       <c r="B202" s="1"/>
       <c r="C202" s="41"/>
       <c r="D202" s="42">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E202" s="43">
-        <v>2362</v>
+        <v>5284</v>
       </c>
       <c r="F202" s="33"/>
       <c r="G202" s="2"/>
@@ -3904,10 +3904,10 @@
       <c r="B203" s="1"/>
       <c r="C203" s="41"/>
       <c r="D203" s="42">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E203" s="43">
-        <v>2709</v>
+        <v>2362</v>
       </c>
       <c r="F203" s="33"/>
       <c r="G203" s="2"/>
@@ -3917,10 +3917,10 @@
       <c r="B204" s="1"/>
       <c r="C204" s="41"/>
       <c r="D204" s="42">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E204" s="43">
-        <v>1213</v>
+        <v>2709</v>
       </c>
       <c r="F204" s="33"/>
       <c r="G204" s="2"/>
@@ -3930,10 +3930,10 @@
       <c r="B205" s="1"/>
       <c r="C205" s="41"/>
       <c r="D205" s="42">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E205" s="43">
-        <v>3597</v>
+        <v>1213</v>
       </c>
       <c r="F205" s="33"/>
       <c r="G205" s="2"/>
@@ -3943,10 +3943,10 @@
       <c r="B206" s="1"/>
       <c r="C206" s="41"/>
       <c r="D206" s="42">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E206" s="43">
-        <v>5548</v>
+        <v>3597</v>
       </c>
       <c r="F206" s="33"/>
       <c r="G206" s="2"/>
@@ -3956,10 +3956,10 @@
       <c r="B207" s="1"/>
       <c r="C207" s="41"/>
       <c r="D207" s="42">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E207" s="43">
-        <v>9423</v>
+        <v>5548</v>
       </c>
       <c r="F207" s="33"/>
       <c r="G207" s="2"/>
@@ -3969,10 +3969,10 @@
       <c r="B208" s="1"/>
       <c r="C208" s="41"/>
       <c r="D208" s="42">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E208" s="43">
-        <v>9378</v>
+        <v>9423</v>
       </c>
       <c r="F208" s="33"/>
       <c r="G208" s="2"/>
@@ -3982,10 +3982,10 @@
       <c r="B209" s="1"/>
       <c r="C209" s="41"/>
       <c r="D209" s="42">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E209" s="43">
-        <v>5655</v>
+        <v>9378</v>
       </c>
       <c r="F209" s="33"/>
       <c r="G209" s="2"/>
@@ -3995,10 +3995,10 @@
       <c r="B210" s="1"/>
       <c r="C210" s="41"/>
       <c r="D210" s="42">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E210" s="43">
-        <v>7434</v>
+        <v>5655</v>
       </c>
       <c r="F210" s="33"/>
       <c r="G210" s="2"/>
@@ -4008,10 +4008,10 @@
       <c r="B211" s="1"/>
       <c r="C211" s="41"/>
       <c r="D211" s="42">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E211" s="43">
-        <v>2593</v>
+        <v>7434</v>
       </c>
       <c r="F211" s="33"/>
       <c r="G211" s="2"/>
@@ -4021,10 +4021,10 @@
       <c r="B212" s="1"/>
       <c r="C212" s="41"/>
       <c r="D212" s="42">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E212" s="43">
-        <v>3126</v>
+        <v>2593</v>
       </c>
       <c r="F212" s="33"/>
       <c r="G212" s="2"/>
@@ -4034,10 +4034,10 @@
       <c r="B213" s="1"/>
       <c r="C213" s="41"/>
       <c r="D213" s="42">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E213" s="43">
-        <v>2792</v>
+        <v>3126</v>
       </c>
       <c r="F213" s="33"/>
       <c r="G213" s="2"/>
@@ -4047,10 +4047,10 @@
       <c r="B214" s="1"/>
       <c r="C214" s="41"/>
       <c r="D214" s="42">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E214" s="43">
-        <v>966</v>
+        <v>2792</v>
       </c>
       <c r="F214" s="33"/>
       <c r="G214" s="2"/>
@@ -4060,10 +4060,10 @@
       <c r="B215" s="1"/>
       <c r="C215" s="41"/>
       <c r="D215" s="42">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E215" s="43">
-        <v>1885</v>
+        <v>966</v>
       </c>
       <c r="F215" s="33"/>
       <c r="G215" s="2"/>
@@ -4073,10 +4073,10 @@
       <c r="B216" s="1"/>
       <c r="C216" s="41"/>
       <c r="D216" s="42">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E216" s="43">
-        <v>2233</v>
+        <v>1885</v>
       </c>
       <c r="F216" s="33"/>
       <c r="G216" s="2"/>
@@ -4086,10 +4086,10 @@
       <c r="B217" s="1"/>
       <c r="C217" s="41"/>
       <c r="D217" s="42">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E217" s="43">
-        <v>646</v>
+        <v>2233</v>
       </c>
       <c r="F217" s="33"/>
       <c r="G217" s="2"/>
@@ -4099,10 +4099,10 @@
       <c r="B218" s="1"/>
       <c r="C218" s="41"/>
       <c r="D218" s="42">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E218" s="43">
-        <v>212</v>
+        <v>646</v>
       </c>
       <c r="F218" s="33"/>
       <c r="G218" s="2"/>
@@ -4112,10 +4112,10 @@
       <c r="B219" s="1"/>
       <c r="C219" s="41"/>
       <c r="D219" s="42">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E219" s="43">
-        <v>278</v>
+        <v>212</v>
       </c>
       <c r="F219" s="33"/>
       <c r="G219" s="2"/>
@@ -4123,12 +4123,12 @@
     </row>
     <row r="220" spans="2:8" ht="18.75" customHeight="1">
       <c r="B220" s="1"/>
-      <c r="C220" s="60"/>
-      <c r="D220" s="61">
-        <v>196</v>
-      </c>
-      <c r="E220" s="64">
-        <v>70</v>
+      <c r="C220" s="41"/>
+      <c r="D220" s="42">
+        <v>195</v>
+      </c>
+      <c r="E220" s="43">
+        <v>278</v>
       </c>
       <c r="F220" s="33"/>
       <c r="G220" s="2"/>
@@ -4136,14 +4136,12 @@
     </row>
     <row r="221" spans="2:8" ht="18.75" customHeight="1">
       <c r="B221" s="1"/>
-      <c r="C221" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="D221" s="63">
-        <v>1</v>
-      </c>
-      <c r="E221" s="65">
-        <v>166</v>
+      <c r="C221" s="60"/>
+      <c r="D221" s="61">
+        <v>196</v>
+      </c>
+      <c r="E221" s="64">
+        <v>70</v>
       </c>
       <c r="F221" s="33"/>
       <c r="G221" s="2"/>
@@ -4151,14 +4149,14 @@
     </row>
     <row r="222" spans="2:8" ht="18.75" customHeight="1">
       <c r="B222" s="1"/>
-      <c r="C222" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="D222" s="42">
-        <v>2</v>
-      </c>
-      <c r="E222" s="43">
-        <v>2031</v>
+      <c r="C222" s="62" t="s">
+        <v>22</v>
+      </c>
+      <c r="D222" s="63">
+        <v>1</v>
+      </c>
+      <c r="E222" s="65">
+        <v>166</v>
       </c>
       <c r="F222" s="33"/>
       <c r="G222" s="2"/>
@@ -4166,12 +4164,14 @@
     </row>
     <row r="223" spans="2:8" ht="18.75" customHeight="1">
       <c r="B223" s="1"/>
-      <c r="C223" s="41"/>
+      <c r="C223" s="41" t="s">
+        <v>33</v>
+      </c>
       <c r="D223" s="42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E223" s="43">
-        <v>2580</v>
+        <v>2031</v>
       </c>
       <c r="F223" s="33"/>
       <c r="G223" s="2"/>
@@ -4181,10 +4181,10 @@
       <c r="B224" s="1"/>
       <c r="C224" s="41"/>
       <c r="D224" s="42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E224" s="43">
-        <v>6481</v>
+        <v>2580</v>
       </c>
       <c r="F224" s="33"/>
       <c r="G224" s="2"/>
@@ -4194,10 +4194,10 @@
       <c r="B225" s="1"/>
       <c r="C225" s="41"/>
       <c r="D225" s="42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E225" s="43">
-        <v>2203</v>
+        <v>6481</v>
       </c>
       <c r="F225" s="33"/>
       <c r="G225" s="2"/>
@@ -4207,10 +4207,10 @@
       <c r="B226" s="1"/>
       <c r="C226" s="41"/>
       <c r="D226" s="42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E226" s="43">
-        <v>4675</v>
+        <v>2203</v>
       </c>
       <c r="F226" s="33"/>
       <c r="G226" s="2"/>
@@ -4220,10 +4220,10 @@
       <c r="B227" s="1"/>
       <c r="C227" s="41"/>
       <c r="D227" s="42">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E227" s="43">
-        <v>3290</v>
+        <v>4675</v>
       </c>
       <c r="F227" s="33"/>
       <c r="G227" s="2"/>
@@ -4233,10 +4233,10 @@
       <c r="B228" s="1"/>
       <c r="C228" s="41"/>
       <c r="D228" s="42">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E228" s="43">
-        <v>2322</v>
+        <v>3290</v>
       </c>
       <c r="F228" s="33"/>
       <c r="G228" s="2"/>
@@ -4246,10 +4246,10 @@
       <c r="B229" s="1"/>
       <c r="C229" s="41"/>
       <c r="D229" s="42">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E229" s="43">
-        <v>2831</v>
+        <v>2322</v>
       </c>
       <c r="F229" s="33"/>
       <c r="G229" s="2"/>
@@ -4259,10 +4259,10 @@
       <c r="B230" s="1"/>
       <c r="C230" s="41"/>
       <c r="D230" s="42">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E230" s="43">
-        <v>5106</v>
+        <v>2831</v>
       </c>
       <c r="F230" s="33"/>
       <c r="G230" s="2"/>
@@ -4272,10 +4272,10 @@
       <c r="B231" s="1"/>
       <c r="C231" s="41"/>
       <c r="D231" s="42">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E231" s="43">
-        <v>3169</v>
+        <v>5106</v>
       </c>
       <c r="F231" s="33"/>
       <c r="G231" s="2"/>
@@ -4285,10 +4285,10 @@
       <c r="B232" s="1"/>
       <c r="C232" s="41"/>
       <c r="D232" s="42">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E232" s="43">
-        <v>3055</v>
+        <v>3169</v>
       </c>
       <c r="F232" s="33"/>
       <c r="G232" s="2"/>
@@ -4298,10 +4298,10 @@
       <c r="B233" s="1"/>
       <c r="C233" s="41"/>
       <c r="D233" s="42">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E233" s="43">
-        <v>1826</v>
+        <v>3055</v>
       </c>
       <c r="F233" s="33"/>
       <c r="G233" s="2"/>
@@ -4311,10 +4311,10 @@
       <c r="B234" s="1"/>
       <c r="C234" s="41"/>
       <c r="D234" s="42">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E234" s="43">
-        <v>3532</v>
+        <v>1826</v>
       </c>
       <c r="F234" s="33"/>
       <c r="G234" s="2"/>
@@ -4324,10 +4324,10 @@
       <c r="B235" s="1"/>
       <c r="C235" s="41"/>
       <c r="D235" s="42">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E235" s="43">
-        <v>3892</v>
+        <v>3532</v>
       </c>
       <c r="F235" s="33"/>
       <c r="G235" s="2"/>
@@ -4337,10 +4337,10 @@
       <c r="B236" s="1"/>
       <c r="C236" s="41"/>
       <c r="D236" s="42">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E236" s="43">
-        <v>4024</v>
+        <v>3892</v>
       </c>
       <c r="F236" s="33"/>
       <c r="G236" s="2"/>
@@ -4350,10 +4350,10 @@
       <c r="B237" s="1"/>
       <c r="C237" s="41"/>
       <c r="D237" s="42">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E237" s="43">
-        <v>3789</v>
+        <v>4024</v>
       </c>
       <c r="F237" s="33"/>
       <c r="G237" s="2"/>
@@ -4363,10 +4363,10 @@
       <c r="B238" s="1"/>
       <c r="C238" s="41"/>
       <c r="D238" s="42">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E238" s="43">
-        <v>1965</v>
+        <v>3789</v>
       </c>
       <c r="F238" s="33"/>
       <c r="G238" s="2"/>
@@ -4376,10 +4376,10 @@
       <c r="B239" s="1"/>
       <c r="C239" s="41"/>
       <c r="D239" s="42">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E239" s="43">
-        <v>2749</v>
+        <v>1965</v>
       </c>
       <c r="F239" s="33"/>
       <c r="G239" s="2"/>
@@ -4389,10 +4389,10 @@
       <c r="B240" s="1"/>
       <c r="C240" s="41"/>
       <c r="D240" s="42">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E240" s="43">
-        <v>3464</v>
+        <v>2749</v>
       </c>
       <c r="F240" s="33"/>
       <c r="G240" s="2"/>
@@ -4402,10 +4402,10 @@
       <c r="B241" s="1"/>
       <c r="C241" s="41"/>
       <c r="D241" s="42">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E241" s="43">
-        <v>2557</v>
+        <v>3464</v>
       </c>
       <c r="F241" s="33"/>
       <c r="G241" s="2"/>
@@ -4415,10 +4415,10 @@
       <c r="B242" s="1"/>
       <c r="C242" s="41"/>
       <c r="D242" s="42">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E242" s="43">
-        <v>2601</v>
+        <v>2557</v>
       </c>
       <c r="F242" s="33"/>
       <c r="G242" s="2"/>
@@ -4428,10 +4428,10 @@
       <c r="B243" s="1"/>
       <c r="C243" s="41"/>
       <c r="D243" s="42">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E243" s="43">
-        <v>3489</v>
+        <v>2601</v>
       </c>
       <c r="F243" s="33"/>
       <c r="G243" s="2"/>
@@ -4441,10 +4441,10 @@
       <c r="B244" s="1"/>
       <c r="C244" s="41"/>
       <c r="D244" s="42">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E244" s="43">
-        <v>3429</v>
+        <v>3489</v>
       </c>
       <c r="F244" s="33"/>
       <c r="G244" s="2"/>
@@ -4454,10 +4454,10 @@
       <c r="B245" s="1"/>
       <c r="C245" s="41"/>
       <c r="D245" s="42">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E245" s="43">
-        <v>2997</v>
+        <v>3429</v>
       </c>
       <c r="F245" s="33"/>
       <c r="G245" s="2"/>
@@ -4467,10 +4467,10 @@
       <c r="B246" s="1"/>
       <c r="C246" s="41"/>
       <c r="D246" s="42">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E246" s="43">
-        <v>3523</v>
+        <v>3025</v>
       </c>
       <c r="F246" s="33"/>
       <c r="G246" s="2"/>
@@ -4480,10 +4480,10 @@
       <c r="B247" s="1"/>
       <c r="C247" s="41"/>
       <c r="D247" s="42">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E247" s="43">
-        <v>3481</v>
+        <v>3646</v>
       </c>
       <c r="F247" s="33"/>
       <c r="G247" s="2"/>
@@ -4493,10 +4493,10 @@
       <c r="B248" s="1"/>
       <c r="C248" s="41"/>
       <c r="D248" s="42">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E248" s="43">
-        <v>2721</v>
+        <v>3481</v>
       </c>
       <c r="F248" s="33"/>
       <c r="G248" s="2"/>
@@ -4506,10 +4506,10 @@
       <c r="B249" s="1"/>
       <c r="C249" s="41"/>
       <c r="D249" s="42">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E249" s="43">
-        <v>4972</v>
+        <v>2721</v>
       </c>
       <c r="F249" s="33"/>
       <c r="G249" s="2"/>
@@ -4519,10 +4519,10 @@
       <c r="B250" s="1"/>
       <c r="C250" s="41"/>
       <c r="D250" s="42">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E250" s="43">
-        <v>2913</v>
+        <v>4972</v>
       </c>
       <c r="F250" s="33"/>
       <c r="G250" s="2"/>
@@ -4532,10 +4532,10 @@
       <c r="B251" s="1"/>
       <c r="C251" s="41"/>
       <c r="D251" s="42">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E251" s="43">
-        <v>3604</v>
+        <v>2913</v>
       </c>
       <c r="F251" s="33"/>
       <c r="G251" s="2"/>
@@ -4545,10 +4545,10 @@
       <c r="B252" s="1"/>
       <c r="C252" s="41"/>
       <c r="D252" s="42">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E252" s="43">
-        <v>4888</v>
+        <v>3604</v>
       </c>
       <c r="F252" s="33"/>
       <c r="G252" s="2"/>
@@ -4558,10 +4558,10 @@
       <c r="B253" s="1"/>
       <c r="C253" s="41"/>
       <c r="D253" s="42">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E253" s="43">
-        <v>6083</v>
+        <v>4888</v>
       </c>
       <c r="F253" s="33"/>
       <c r="G253" s="2"/>
@@ -4571,10 +4571,10 @@
       <c r="B254" s="1"/>
       <c r="C254" s="41"/>
       <c r="D254" s="42">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E254" s="43">
-        <v>5436</v>
+        <v>6091</v>
       </c>
       <c r="F254" s="33"/>
       <c r="G254" s="2"/>
@@ -4584,10 +4584,10 @@
       <c r="B255" s="1"/>
       <c r="C255" s="41"/>
       <c r="D255" s="42">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E255" s="43">
-        <v>5960</v>
+        <v>5436</v>
       </c>
       <c r="F255" s="33"/>
       <c r="G255" s="2"/>
@@ -4597,10 +4597,10 @@
       <c r="B256" s="1"/>
       <c r="C256" s="41"/>
       <c r="D256" s="42">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E256" s="43">
-        <v>7713</v>
+        <v>5960</v>
       </c>
       <c r="F256" s="33"/>
       <c r="G256" s="2"/>
@@ -4610,10 +4610,10 @@
       <c r="B257" s="1"/>
       <c r="C257" s="41"/>
       <c r="D257" s="42">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E257" s="43">
-        <v>2823</v>
+        <v>7713</v>
       </c>
       <c r="F257" s="33"/>
       <c r="G257" s="2"/>
@@ -4623,10 +4623,10 @@
       <c r="B258" s="1"/>
       <c r="C258" s="41"/>
       <c r="D258" s="42">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E258" s="43">
-        <v>5496</v>
+        <v>2823</v>
       </c>
       <c r="F258" s="33"/>
       <c r="G258" s="2"/>
@@ -4636,10 +4636,10 @@
       <c r="B259" s="1"/>
       <c r="C259" s="41"/>
       <c r="D259" s="42">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E259" s="43">
-        <v>6375</v>
+        <v>5496</v>
       </c>
       <c r="F259" s="33"/>
       <c r="G259" s="2"/>
@@ -4649,10 +4649,10 @@
       <c r="B260" s="1"/>
       <c r="C260" s="41"/>
       <c r="D260" s="42">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E260" s="43">
-        <v>6537</v>
+        <v>6375</v>
       </c>
       <c r="F260" s="33"/>
       <c r="G260" s="2"/>
@@ -4662,10 +4662,10 @@
       <c r="B261" s="1"/>
       <c r="C261" s="41"/>
       <c r="D261" s="42">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E261" s="43">
-        <v>6915</v>
+        <v>6537</v>
       </c>
       <c r="F261" s="33"/>
       <c r="G261" s="2"/>
@@ -4675,10 +4675,10 @@
       <c r="B262" s="1"/>
       <c r="C262" s="41"/>
       <c r="D262" s="42">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E262" s="43">
-        <v>6374</v>
+        <v>6915</v>
       </c>
       <c r="F262" s="33"/>
       <c r="G262" s="2"/>
@@ -4688,10 +4688,10 @@
       <c r="B263" s="1"/>
       <c r="C263" s="41"/>
       <c r="D263" s="42">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E263" s="43">
-        <v>10306</v>
+        <v>6374</v>
       </c>
       <c r="F263" s="33"/>
       <c r="G263" s="2"/>
@@ -4701,10 +4701,10 @@
       <c r="B264" s="1"/>
       <c r="C264" s="41"/>
       <c r="D264" s="42">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E264" s="43">
-        <v>9761</v>
+        <v>10306</v>
       </c>
       <c r="F264" s="33"/>
       <c r="G264" s="2"/>
@@ -4714,10 +4714,10 @@
       <c r="B265" s="1"/>
       <c r="C265" s="41"/>
       <c r="D265" s="42">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E265" s="43">
-        <v>15347</v>
+        <v>9761</v>
       </c>
       <c r="F265" s="33"/>
       <c r="G265" s="2"/>
@@ -4727,10 +4727,10 @@
       <c r="B266" s="1"/>
       <c r="C266" s="41"/>
       <c r="D266" s="42">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E266" s="43">
-        <v>14157</v>
+        <v>15347</v>
       </c>
       <c r="F266" s="33"/>
       <c r="G266" s="2"/>
@@ -4740,10 +4740,10 @@
       <c r="B267" s="1"/>
       <c r="C267" s="41"/>
       <c r="D267" s="42">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E267" s="43">
-        <v>20127</v>
+        <v>14157</v>
       </c>
       <c r="F267" s="33"/>
       <c r="G267" s="2"/>
@@ -4753,10 +4753,10 @@
       <c r="B268" s="1"/>
       <c r="C268" s="41"/>
       <c r="D268" s="42">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E268" s="43">
-        <v>22038</v>
+        <v>20127</v>
       </c>
       <c r="F268" s="33"/>
       <c r="G268" s="2"/>
@@ -4766,10 +4766,10 @@
       <c r="B269" s="1"/>
       <c r="C269" s="41"/>
       <c r="D269" s="42">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E269" s="43">
-        <v>19608</v>
+        <v>22038</v>
       </c>
       <c r="F269" s="33"/>
       <c r="G269" s="2"/>
@@ -4779,10 +4779,10 @@
       <c r="B270" s="1"/>
       <c r="C270" s="41"/>
       <c r="D270" s="42">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E270" s="43">
-        <v>13064</v>
+        <v>19608</v>
       </c>
       <c r="F270" s="33"/>
       <c r="G270" s="2"/>
@@ -4792,10 +4792,10 @@
       <c r="B271" s="1"/>
       <c r="C271" s="41"/>
       <c r="D271" s="42">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E271" s="43">
-        <v>16097</v>
+        <v>13064</v>
       </c>
       <c r="F271" s="33"/>
       <c r="G271" s="2"/>
@@ -4805,10 +4805,10 @@
       <c r="B272" s="1"/>
       <c r="C272" s="41"/>
       <c r="D272" s="42">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E272" s="43">
-        <v>12505</v>
+        <v>16097</v>
       </c>
       <c r="F272" s="33"/>
       <c r="G272" s="2"/>
@@ -4818,10 +4818,10 @@
       <c r="B273" s="1"/>
       <c r="C273" s="41"/>
       <c r="D273" s="42">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E273" s="43">
-        <v>13110</v>
+        <v>12505</v>
       </c>
       <c r="F273" s="33"/>
       <c r="G273" s="2"/>
@@ -4831,10 +4831,10 @@
       <c r="B274" s="1"/>
       <c r="C274" s="41"/>
       <c r="D274" s="42">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E274" s="43">
-        <v>14769</v>
+        <v>13110</v>
       </c>
       <c r="F274" s="33"/>
       <c r="G274" s="2"/>
@@ -4844,10 +4844,10 @@
       <c r="B275" s="1"/>
       <c r="C275" s="41"/>
       <c r="D275" s="42">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E275" s="43">
-        <v>12382</v>
+        <v>14769</v>
       </c>
       <c r="F275" s="33"/>
       <c r="G275" s="2"/>
@@ -4857,10 +4857,10 @@
       <c r="B276" s="1"/>
       <c r="C276" s="41"/>
       <c r="D276" s="42">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E276" s="43">
-        <v>11837</v>
+        <v>12382</v>
       </c>
       <c r="F276" s="33"/>
       <c r="G276" s="2"/>
@@ -4870,10 +4870,10 @@
       <c r="B277" s="1"/>
       <c r="C277" s="41"/>
       <c r="D277" s="42">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E277" s="43">
-        <v>11776</v>
+        <v>11837</v>
       </c>
       <c r="F277" s="33"/>
       <c r="G277" s="2"/>
@@ -4883,10 +4883,10 @@
       <c r="B278" s="1"/>
       <c r="C278" s="41"/>
       <c r="D278" s="42">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E278" s="43">
-        <v>19457</v>
+        <v>11776</v>
       </c>
       <c r="F278" s="33"/>
       <c r="G278" s="2"/>
@@ -4896,10 +4896,10 @@
       <c r="B279" s="1"/>
       <c r="C279" s="41"/>
       <c r="D279" s="42">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E279" s="43">
-        <v>5695</v>
+        <v>19457</v>
       </c>
       <c r="F279" s="33"/>
       <c r="G279" s="2"/>
@@ -4909,10 +4909,10 @@
       <c r="B280" s="1"/>
       <c r="C280" s="41"/>
       <c r="D280" s="42">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E280" s="43">
-        <v>11992</v>
+        <v>5695</v>
       </c>
       <c r="F280" s="33"/>
       <c r="G280" s="2"/>
@@ -4922,10 +4922,10 @@
       <c r="B281" s="1"/>
       <c r="C281" s="41"/>
       <c r="D281" s="42">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E281" s="43">
-        <v>7193</v>
+        <v>11992</v>
       </c>
       <c r="F281" s="33"/>
       <c r="G281" s="2"/>
@@ -4935,10 +4935,10 @@
       <c r="B282" s="1"/>
       <c r="C282" s="41"/>
       <c r="D282" s="42">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E282" s="43">
-        <v>7062</v>
+        <v>7193</v>
       </c>
       <c r="F282" s="33"/>
       <c r="G282" s="2"/>
@@ -4948,10 +4948,10 @@
       <c r="B283" s="1"/>
       <c r="C283" s="41"/>
       <c r="D283" s="42">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E283" s="43">
-        <v>12937</v>
+        <v>7062</v>
       </c>
       <c r="F283" s="33"/>
       <c r="G283" s="2"/>
@@ -4961,10 +4961,10 @@
       <c r="B284" s="1"/>
       <c r="C284" s="41"/>
       <c r="D284" s="42">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E284" s="43">
-        <v>12274</v>
+        <v>12937</v>
       </c>
       <c r="F284" s="33"/>
       <c r="G284" s="2"/>
@@ -4974,10 +4974,10 @@
       <c r="B285" s="1"/>
       <c r="C285" s="41"/>
       <c r="D285" s="42">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E285" s="43">
-        <v>3231</v>
+        <v>12274</v>
       </c>
       <c r="F285" s="33"/>
       <c r="G285" s="2"/>
@@ -4987,10 +4987,10 @@
       <c r="B286" s="1"/>
       <c r="C286" s="41"/>
       <c r="D286" s="42">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E286" s="43">
-        <v>4468</v>
+        <v>3231</v>
       </c>
       <c r="F286" s="33"/>
       <c r="G286" s="2"/>
@@ -5000,10 +5000,10 @@
       <c r="B287" s="1"/>
       <c r="C287" s="41"/>
       <c r="D287" s="42">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E287" s="43">
-        <v>9466</v>
+        <v>4468</v>
       </c>
       <c r="F287" s="33"/>
       <c r="G287" s="2"/>
@@ -5013,10 +5013,10 @@
       <c r="B288" s="1"/>
       <c r="C288" s="41"/>
       <c r="D288" s="42">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E288" s="43">
-        <v>6084</v>
+        <v>9466</v>
       </c>
       <c r="F288" s="33"/>
       <c r="G288" s="2"/>
@@ -5026,10 +5026,10 @@
       <c r="B289" s="1"/>
       <c r="C289" s="41"/>
       <c r="D289" s="42">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E289" s="43">
-        <v>2258</v>
+        <v>6084</v>
       </c>
       <c r="F289" s="33"/>
       <c r="G289" s="2"/>
@@ -5039,10 +5039,10 @@
       <c r="B290" s="1"/>
       <c r="C290" s="41"/>
       <c r="D290" s="42">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E290" s="43">
-        <v>3297</v>
+        <v>2258</v>
       </c>
       <c r="F290" s="33"/>
       <c r="G290" s="2"/>
@@ -5052,10 +5052,10 @@
       <c r="B291" s="1"/>
       <c r="C291" s="41"/>
       <c r="D291" s="42">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E291" s="43">
-        <v>6029</v>
+        <v>3597</v>
       </c>
       <c r="F291" s="33"/>
       <c r="G291" s="2"/>
@@ -5065,10 +5065,10 @@
       <c r="B292" s="1"/>
       <c r="C292" s="41"/>
       <c r="D292" s="42">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E292" s="43">
-        <v>2524</v>
+        <v>6029</v>
       </c>
       <c r="F292" s="33"/>
       <c r="G292" s="2"/>
@@ -5078,10 +5078,10 @@
       <c r="B293" s="1"/>
       <c r="C293" s="41"/>
       <c r="D293" s="42">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E293" s="43">
-        <v>2473</v>
+        <v>2524</v>
       </c>
       <c r="F293" s="33"/>
       <c r="G293" s="2"/>
@@ -5091,10 +5091,10 @@
       <c r="B294" s="1"/>
       <c r="C294" s="41"/>
       <c r="D294" s="42">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E294" s="43">
-        <v>2384</v>
+        <v>2473</v>
       </c>
       <c r="F294" s="33"/>
       <c r="G294" s="2"/>
@@ -5104,10 +5104,10 @@
       <c r="B295" s="1"/>
       <c r="C295" s="41"/>
       <c r="D295" s="42">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E295" s="43">
-        <v>3272</v>
+        <v>2384</v>
       </c>
       <c r="F295" s="33"/>
       <c r="G295" s="2"/>
@@ -5117,10 +5117,10 @@
       <c r="B296" s="1"/>
       <c r="C296" s="41"/>
       <c r="D296" s="42">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E296" s="43">
-        <v>2980</v>
+        <v>3272</v>
       </c>
       <c r="F296" s="33"/>
       <c r="G296" s="2"/>
@@ -5130,10 +5130,10 @@
       <c r="B297" s="1"/>
       <c r="C297" s="41"/>
       <c r="D297" s="42">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E297" s="43">
-        <v>5752</v>
+        <v>2980</v>
       </c>
       <c r="F297" s="33"/>
       <c r="G297" s="2"/>
@@ -5143,10 +5143,10 @@
       <c r="B298" s="1"/>
       <c r="C298" s="41"/>
       <c r="D298" s="42">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E298" s="43">
-        <v>3011</v>
+        <v>5752</v>
       </c>
       <c r="F298" s="33"/>
       <c r="G298" s="2"/>
@@ -5156,10 +5156,10 @@
       <c r="B299" s="1"/>
       <c r="C299" s="41"/>
       <c r="D299" s="42">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E299" s="43">
-        <v>1682</v>
+        <v>3011</v>
       </c>
       <c r="F299" s="33"/>
       <c r="G299" s="2"/>
@@ -5169,10 +5169,10 @@
       <c r="B300" s="1"/>
       <c r="C300" s="41"/>
       <c r="D300" s="42">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E300" s="43">
-        <v>3465</v>
+        <v>1682</v>
       </c>
       <c r="F300" s="33"/>
       <c r="G300" s="2"/>
@@ -5182,10 +5182,10 @@
       <c r="B301" s="1"/>
       <c r="C301" s="41"/>
       <c r="D301" s="42">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E301" s="43">
-        <v>3239</v>
+        <v>3465</v>
       </c>
       <c r="F301" s="33"/>
       <c r="G301" s="2"/>
@@ -5195,10 +5195,10 @@
       <c r="B302" s="1"/>
       <c r="C302" s="41"/>
       <c r="D302" s="42">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E302" s="43">
-        <v>1167</v>
+        <v>3239</v>
       </c>
       <c r="F302" s="33"/>
       <c r="G302" s="2"/>
@@ -5208,10 +5208,10 @@
       <c r="B303" s="1"/>
       <c r="C303" s="41"/>
       <c r="D303" s="42">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E303" s="43">
-        <v>1889</v>
+        <v>1167</v>
       </c>
       <c r="F303" s="33"/>
       <c r="G303" s="2"/>
@@ -5221,10 +5221,10 @@
       <c r="B304" s="1"/>
       <c r="C304" s="41"/>
       <c r="D304" s="42">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E304" s="43">
-        <v>699</v>
+        <v>1889</v>
       </c>
       <c r="F304" s="33"/>
       <c r="G304" s="2"/>
@@ -5234,10 +5234,10 @@
       <c r="B305" s="1"/>
       <c r="C305" s="41"/>
       <c r="D305" s="42">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E305" s="43">
-        <v>716</v>
+        <v>699</v>
       </c>
       <c r="F305" s="33"/>
       <c r="G305" s="2"/>
@@ -5247,10 +5247,10 @@
       <c r="B306" s="1"/>
       <c r="C306" s="41"/>
       <c r="D306" s="42">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E306" s="43">
-        <v>407</v>
+        <v>716</v>
       </c>
       <c r="F306" s="33"/>
       <c r="G306" s="2"/>
@@ -5260,10 +5260,10 @@
       <c r="B307" s="1"/>
       <c r="C307" s="41"/>
       <c r="D307" s="42">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E307" s="43">
-        <v>261</v>
+        <v>407</v>
       </c>
       <c r="F307" s="33"/>
       <c r="G307" s="2"/>
@@ -5273,10 +5273,10 @@
       <c r="B308" s="1"/>
       <c r="C308" s="41"/>
       <c r="D308" s="42">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E308" s="43">
-        <v>342</v>
+        <v>261</v>
       </c>
       <c r="F308" s="33"/>
       <c r="G308" s="2"/>
@@ -5286,10 +5286,10 @@
       <c r="B309" s="1"/>
       <c r="C309" s="41"/>
       <c r="D309" s="42">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E309" s="43">
-        <v>573</v>
+        <v>342</v>
       </c>
       <c r="F309" s="33"/>
       <c r="G309" s="2"/>
@@ -5299,10 +5299,10 @@
       <c r="B310" s="1"/>
       <c r="C310" s="41"/>
       <c r="D310" s="42">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E310" s="43">
-        <v>246</v>
+        <v>573</v>
       </c>
       <c r="F310" s="33"/>
       <c r="G310" s="2"/>
@@ -5310,12 +5310,12 @@
     </row>
     <row r="311" spans="2:8" ht="18.75" customHeight="1">
       <c r="B311" s="1"/>
-      <c r="C311" s="60"/>
-      <c r="D311" s="61">
-        <v>91</v>
-      </c>
-      <c r="E311" s="64">
-        <v>265</v>
+      <c r="C311" s="41"/>
+      <c r="D311" s="42">
+        <v>90</v>
+      </c>
+      <c r="E311" s="43">
+        <v>246</v>
       </c>
       <c r="F311" s="33"/>
       <c r="G311" s="2"/>
@@ -5323,14 +5323,12 @@
     </row>
     <row r="312" spans="2:8" ht="18.75" customHeight="1">
       <c r="B312" s="1"/>
-      <c r="C312" s="62" t="s">
-        <v>23</v>
-      </c>
-      <c r="D312" s="63">
-        <v>1</v>
-      </c>
-      <c r="E312" s="65">
-        <v>4447</v>
+      <c r="C312" s="60"/>
+      <c r="D312" s="61">
+        <v>91</v>
+      </c>
+      <c r="E312" s="64">
+        <v>265</v>
       </c>
       <c r="F312" s="33"/>
       <c r="G312" s="2"/>
@@ -5338,14 +5336,14 @@
     </row>
     <row r="313" spans="2:8" ht="18.75" customHeight="1">
       <c r="B313" s="1"/>
-      <c r="C313" s="41" t="s">
-        <v>34</v>
-      </c>
-      <c r="D313" s="42">
-        <v>2</v>
-      </c>
-      <c r="E313" s="43">
-        <v>1633</v>
+      <c r="C313" s="62" t="s">
+        <v>23</v>
+      </c>
+      <c r="D313" s="63">
+        <v>1</v>
+      </c>
+      <c r="E313" s="65">
+        <v>4447</v>
       </c>
       <c r="F313" s="33"/>
       <c r="G313" s="2"/>
@@ -5353,12 +5351,14 @@
     </row>
     <row r="314" spans="2:8" ht="18.75" customHeight="1">
       <c r="B314" s="1"/>
-      <c r="C314" s="41"/>
+      <c r="C314" s="41" t="s">
+        <v>34</v>
+      </c>
       <c r="D314" s="42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E314" s="43">
-        <v>3468</v>
+        <v>1633</v>
       </c>
       <c r="F314" s="33"/>
       <c r="G314" s="2"/>
@@ -5368,10 +5368,10 @@
       <c r="B315" s="1"/>
       <c r="C315" s="41"/>
       <c r="D315" s="42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E315" s="43">
-        <v>3297</v>
+        <v>3468</v>
       </c>
       <c r="F315" s="33"/>
       <c r="G315" s="2"/>
@@ -5381,10 +5381,10 @@
       <c r="B316" s="1"/>
       <c r="C316" s="41"/>
       <c r="D316" s="42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E316" s="43">
-        <v>2172</v>
+        <v>3297</v>
       </c>
       <c r="F316" s="33"/>
       <c r="G316" s="2"/>
@@ -5394,10 +5394,10 @@
       <c r="B317" s="1"/>
       <c r="C317" s="41"/>
       <c r="D317" s="42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E317" s="43">
-        <v>9681</v>
+        <v>2172</v>
       </c>
       <c r="F317" s="33"/>
       <c r="G317" s="2"/>
@@ -5407,10 +5407,10 @@
       <c r="B318" s="1"/>
       <c r="C318" s="41"/>
       <c r="D318" s="42">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E318" s="43">
-        <v>11209</v>
+        <v>9681</v>
       </c>
       <c r="F318" s="33"/>
       <c r="G318" s="2"/>
@@ -5420,10 +5420,10 @@
       <c r="B319" s="1"/>
       <c r="C319" s="41"/>
       <c r="D319" s="42">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E319" s="43">
-        <v>13239</v>
+        <v>11209</v>
       </c>
       <c r="F319" s="33"/>
       <c r="G319" s="2"/>
@@ -5433,10 +5433,10 @@
       <c r="B320" s="1"/>
       <c r="C320" s="41"/>
       <c r="D320" s="42">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E320" s="43">
-        <v>15915</v>
+        <v>13239</v>
       </c>
       <c r="F320" s="33"/>
       <c r="G320" s="2"/>
@@ -5446,10 +5446,10 @@
       <c r="B321" s="1"/>
       <c r="C321" s="41"/>
       <c r="D321" s="42">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E321" s="43">
-        <v>12421</v>
+        <v>15915</v>
       </c>
       <c r="F321" s="33"/>
       <c r="G321" s="2"/>
@@ -5459,10 +5459,10 @@
       <c r="B322" s="1"/>
       <c r="C322" s="41"/>
       <c r="D322" s="42">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E322" s="43">
-        <v>6413</v>
+        <v>12421</v>
       </c>
       <c r="F322" s="33"/>
       <c r="G322" s="2"/>
@@ -5472,10 +5472,10 @@
       <c r="B323" s="1"/>
       <c r="C323" s="41"/>
       <c r="D323" s="42">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E323" s="43">
-        <v>4773</v>
+        <v>6413</v>
       </c>
       <c r="F323" s="33"/>
       <c r="G323" s="2"/>
@@ -5485,10 +5485,10 @@
       <c r="B324" s="1"/>
       <c r="C324" s="41"/>
       <c r="D324" s="42">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E324" s="43">
-        <v>1234</v>
+        <v>4773</v>
       </c>
       <c r="F324" s="33"/>
       <c r="G324" s="2"/>
@@ -5498,10 +5498,10 @@
       <c r="B325" s="1"/>
       <c r="C325" s="41"/>
       <c r="D325" s="42">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E325" s="43">
-        <v>3220</v>
+        <v>1234</v>
       </c>
       <c r="F325" s="33"/>
       <c r="G325" s="2"/>
@@ -5511,10 +5511,10 @@
       <c r="B326" s="1"/>
       <c r="C326" s="41"/>
       <c r="D326" s="42">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E326" s="43">
-        <v>10055</v>
+        <v>3220</v>
       </c>
       <c r="F326" s="33"/>
       <c r="G326" s="2"/>
@@ -5524,10 +5524,10 @@
       <c r="B327" s="1"/>
       <c r="C327" s="41"/>
       <c r="D327" s="42">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E327" s="43">
-        <v>6632</v>
+        <v>10055</v>
       </c>
       <c r="F327" s="33"/>
       <c r="G327" s="2"/>
@@ -5537,10 +5537,10 @@
       <c r="B328" s="1"/>
       <c r="C328" s="41"/>
       <c r="D328" s="42">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E328" s="43">
-        <v>4192</v>
+        <v>6632</v>
       </c>
       <c r="F328" s="33"/>
       <c r="G328" s="2"/>
@@ -5550,10 +5550,10 @@
       <c r="B329" s="1"/>
       <c r="C329" s="41"/>
       <c r="D329" s="42">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E329" s="43">
-        <v>1468</v>
+        <v>4192</v>
       </c>
       <c r="F329" s="33"/>
       <c r="G329" s="2"/>
@@ -5561,12 +5561,12 @@
     </row>
     <row r="330" spans="2:8" ht="18.75" customHeight="1">
       <c r="B330" s="1"/>
-      <c r="C330" s="60"/>
-      <c r="D330" s="61">
-        <v>19</v>
-      </c>
-      <c r="E330" s="64">
-        <v>666</v>
+      <c r="C330" s="41"/>
+      <c r="D330" s="42">
+        <v>18</v>
+      </c>
+      <c r="E330" s="43">
+        <v>1468</v>
       </c>
       <c r="F330" s="33"/>
       <c r="G330" s="2"/>
@@ -5574,14 +5574,12 @@
     </row>
     <row r="331" spans="2:8" ht="18.75" customHeight="1">
       <c r="B331" s="1"/>
-      <c r="C331" s="62" t="s">
-        <v>38</v>
-      </c>
-      <c r="D331" s="63">
-        <v>1</v>
-      </c>
-      <c r="E331" s="65">
-        <v>3210</v>
+      <c r="C331" s="60"/>
+      <c r="D331" s="61">
+        <v>19</v>
+      </c>
+      <c r="E331" s="64">
+        <v>666</v>
       </c>
       <c r="F331" s="33"/>
       <c r="G331" s="2"/>
@@ -5589,14 +5587,14 @@
     </row>
     <row r="332" spans="2:8" ht="18.75" customHeight="1">
       <c r="B332" s="1"/>
-      <c r="C332" s="41" t="s">
-        <v>35</v>
-      </c>
-      <c r="D332" s="42">
-        <v>2</v>
-      </c>
-      <c r="E332" s="43">
-        <v>2732</v>
+      <c r="C332" s="62" t="s">
+        <v>38</v>
+      </c>
+      <c r="D332" s="63">
+        <v>1</v>
+      </c>
+      <c r="E332" s="65">
+        <v>3210</v>
       </c>
       <c r="F332" s="33"/>
       <c r="G332" s="2"/>
@@ -5604,12 +5602,14 @@
     </row>
     <row r="333" spans="2:8" ht="18.75" customHeight="1">
       <c r="B333" s="1"/>
-      <c r="C333" s="41"/>
+      <c r="C333" s="41" t="s">
+        <v>35</v>
+      </c>
       <c r="D333" s="42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E333" s="43">
-        <v>622</v>
+        <v>2732</v>
       </c>
       <c r="F333" s="33"/>
       <c r="G333" s="2"/>
@@ -5619,10 +5619,10 @@
       <c r="B334" s="1"/>
       <c r="C334" s="41"/>
       <c r="D334" s="42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E334" s="43">
-        <v>443</v>
+        <v>622</v>
       </c>
       <c r="F334" s="33"/>
       <c r="G334" s="2"/>
@@ -5630,12 +5630,12 @@
     </row>
     <row r="335" spans="2:8" ht="18.75" customHeight="1">
       <c r="B335" s="1"/>
-      <c r="C335" s="60"/>
-      <c r="D335" s="61">
-        <v>5</v>
-      </c>
-      <c r="E335" s="64">
-        <v>568</v>
+      <c r="C335" s="41"/>
+      <c r="D335" s="42">
+        <v>4</v>
+      </c>
+      <c r="E335" s="43">
+        <v>443</v>
       </c>
       <c r="F335" s="33"/>
       <c r="G335" s="2"/>
@@ -5643,14 +5643,12 @@
     </row>
     <row r="336" spans="2:8" ht="18.75" customHeight="1">
       <c r="B336" s="1"/>
-      <c r="C336" s="62" t="s">
-        <v>39</v>
-      </c>
-      <c r="D336" s="63">
-        <v>1</v>
-      </c>
-      <c r="E336" s="65">
-        <v>3366</v>
+      <c r="C336" s="60"/>
+      <c r="D336" s="61">
+        <v>5</v>
+      </c>
+      <c r="E336" s="64">
+        <v>568</v>
       </c>
       <c r="F336" s="33"/>
       <c r="G336" s="2"/>
@@ -5658,14 +5656,14 @@
     </row>
     <row r="337" spans="2:8" ht="18.75" customHeight="1">
       <c r="B337" s="1"/>
-      <c r="C337" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="D337" s="42">
-        <v>2</v>
-      </c>
-      <c r="E337" s="43">
-        <v>2768</v>
+      <c r="C337" s="62" t="s">
+        <v>39</v>
+      </c>
+      <c r="D337" s="63">
+        <v>1</v>
+      </c>
+      <c r="E337" s="65">
+        <v>3366</v>
       </c>
       <c r="F337" s="33"/>
       <c r="G337" s="2"/>
@@ -5673,12 +5671,14 @@
     </row>
     <row r="338" spans="2:8" ht="18.75" customHeight="1">
       <c r="B338" s="1"/>
-      <c r="C338" s="41"/>
+      <c r="C338" s="41" t="s">
+        <v>36</v>
+      </c>
       <c r="D338" s="42">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E338" s="43">
-        <v>200</v>
+        <v>2768</v>
       </c>
       <c r="F338" s="33"/>
       <c r="G338" s="2"/>
@@ -5688,10 +5688,10 @@
       <c r="B339" s="1"/>
       <c r="C339" s="41"/>
       <c r="D339" s="42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E339" s="43">
-        <v>1220</v>
+        <v>200</v>
       </c>
       <c r="F339" s="8"/>
       <c r="G339" s="2"/>
@@ -5699,12 +5699,12 @@
     </row>
     <row r="340" spans="2:8" ht="18.75" customHeight="1">
       <c r="B340" s="1"/>
-      <c r="C340" s="60"/>
-      <c r="D340" s="61">
-        <v>5</v>
-      </c>
-      <c r="E340" s="64">
-        <v>590</v>
+      <c r="C340" s="41"/>
+      <c r="D340" s="42">
+        <v>4</v>
+      </c>
+      <c r="E340" s="43">
+        <v>1220</v>
       </c>
       <c r="F340" s="8"/>
       <c r="G340" s="2"/>
@@ -5712,14 +5712,12 @@
     </row>
     <row r="341" spans="2:8" ht="18.75" customHeight="1">
       <c r="B341" s="1"/>
-      <c r="C341" s="62" t="s">
-        <v>24</v>
-      </c>
-      <c r="D341" s="63">
-        <v>22</v>
-      </c>
-      <c r="E341" s="65">
-        <v>9279</v>
+      <c r="C341" s="60"/>
+      <c r="D341" s="61">
+        <v>5</v>
+      </c>
+      <c r="E341" s="64">
+        <v>590</v>
       </c>
       <c r="F341" s="8"/>
       <c r="G341" s="2"/>
@@ -5727,14 +5725,14 @@
     </row>
     <row r="342" spans="2:8" ht="18.75" customHeight="1">
       <c r="B342" s="1"/>
-      <c r="C342" s="41" t="s">
-        <v>37</v>
-      </c>
-      <c r="D342" s="42">
-        <v>23</v>
-      </c>
-      <c r="E342" s="43">
-        <v>7920</v>
+      <c r="C342" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="D342" s="63">
+        <v>22</v>
+      </c>
+      <c r="E342" s="65">
+        <v>9279</v>
       </c>
       <c r="F342" s="8"/>
       <c r="G342" s="2"/>
@@ -5742,12 +5740,14 @@
     </row>
     <row r="343" spans="2:8" ht="18.75" customHeight="1">
       <c r="B343" s="1"/>
-      <c r="C343" s="41"/>
+      <c r="C343" s="41" t="s">
+        <v>37</v>
+      </c>
       <c r="D343" s="42">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E343" s="43">
-        <v>5388</v>
+        <v>7920</v>
       </c>
       <c r="F343" s="8"/>
       <c r="G343" s="2"/>
@@ -5757,10 +5757,10 @@
       <c r="B344" s="1"/>
       <c r="C344" s="41"/>
       <c r="D344" s="42">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E344" s="43">
-        <v>4494</v>
+        <v>5388</v>
       </c>
       <c r="F344" s="8"/>
       <c r="G344" s="2"/>
@@ -5770,10 +5770,10 @@
       <c r="B345" s="1"/>
       <c r="C345" s="41"/>
       <c r="D345" s="42">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E345" s="43">
-        <v>5760</v>
+        <v>4494</v>
       </c>
       <c r="F345" s="8"/>
       <c r="G345" s="2"/>
@@ -5783,10 +5783,10 @@
       <c r="B346" s="1"/>
       <c r="C346" s="41"/>
       <c r="D346" s="42">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E346" s="43">
-        <v>5068</v>
+        <v>5760</v>
       </c>
       <c r="F346" s="8"/>
       <c r="G346" s="2"/>
@@ -5796,10 +5796,10 @@
       <c r="B347" s="1"/>
       <c r="C347" s="41"/>
       <c r="D347" s="42">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E347" s="43">
-        <v>4239</v>
+        <v>5068</v>
       </c>
       <c r="F347" s="8"/>
       <c r="G347" s="2"/>
@@ -5809,10 +5809,10 @@
       <c r="B348" s="1"/>
       <c r="C348" s="41"/>
       <c r="D348" s="42">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E348" s="43">
-        <v>1790</v>
+        <v>4239</v>
       </c>
       <c r="F348" s="8"/>
       <c r="G348" s="2"/>
@@ -5822,10 +5822,10 @@
       <c r="B349" s="1"/>
       <c r="C349" s="41"/>
       <c r="D349" s="42">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E349" s="43">
-        <v>2079</v>
+        <v>1790</v>
       </c>
       <c r="F349" s="8"/>
       <c r="G349" s="2"/>
@@ -5833,12 +5833,12 @@
     </row>
     <row r="350" spans="2:8" ht="18.75" customHeight="1">
       <c r="B350" s="1"/>
-      <c r="C350" s="60"/>
-      <c r="D350" s="61">
-        <v>31</v>
-      </c>
-      <c r="E350" s="64">
-        <v>1292</v>
+      <c r="C350" s="41"/>
+      <c r="D350" s="42">
+        <v>30</v>
+      </c>
+      <c r="E350" s="43">
+        <v>2079</v>
       </c>
       <c r="F350" s="8"/>
       <c r="G350" s="2"/>
@@ -5846,6 +5846,13 @@
     </row>
     <row r="351" spans="2:8" ht="18.75" customHeight="1">
       <c r="B351" s="1"/>
+      <c r="C351" s="60"/>
+      <c r="D351" s="61">
+        <v>31</v>
+      </c>
+      <c r="E351" s="64">
+        <v>1292</v>
+      </c>
       <c r="F351" s="8"/>
       <c r="G351" s="2"/>
       <c r="H351" s="1"/>

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-22T08:53Z
</commit_message>
<xml_diff>
--- a/history/jpy/mei_latest.xlsx
+++ b/history/jpy/mei_latest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF7CB05A-4A63-41A8-919E-1EB1A17E14D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473B3F5A-989F-4CE2-B296-66A2DC51D803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1357,7 +1357,7 @@
   <sheetData>
     <row r="3" spans="1:8" ht="18.75" customHeight="1">
       <c r="A3" s="50">
-        <v>46304</v>
+        <v>46315</v>
       </c>
       <c r="B3" s="50"/>
       <c r="C3" s="50"/>
@@ -1368,7 +1368,7 @@
     </row>
     <row r="4" spans="1:8" ht="18.75" customHeight="1">
       <c r="A4" s="51">
-        <v>46304</v>
+        <v>46315</v>
       </c>
       <c r="B4" s="51"/>
       <c r="C4" s="51"/>
@@ -1386,10 +1386,10 @@
     </row>
     <row r="7" spans="1:8" ht="18.75" customHeight="1">
       <c r="B7" s="12">
-        <v>46309</v>
+        <v>46317</v>
       </c>
       <c r="F7" s="29">
-        <v>46309</v>
+        <v>46317</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18.75" customHeight="1">
@@ -2144,7 +2144,7 @@
         <v>178</v>
       </c>
       <c r="E68" s="43">
-        <v>22955</v>
+        <v>23035</v>
       </c>
       <c r="F68" s="33"/>
       <c r="G68" s="2"/>
@@ -2157,7 +2157,7 @@
         <v>179</v>
       </c>
       <c r="E69" s="43">
-        <v>9507</v>
+        <v>9543</v>
       </c>
       <c r="F69" s="33"/>
       <c r="G69" s="2"/>
@@ -2222,7 +2222,7 @@
         <v>184</v>
       </c>
       <c r="E74" s="43">
-        <v>1921</v>
+        <v>2087</v>
       </c>
       <c r="F74" s="33"/>
       <c r="G74" s="2"/>
@@ -2235,7 +2235,7 @@
         <v>185</v>
       </c>
       <c r="E75" s="43">
-        <v>5493</v>
+        <v>5863</v>
       </c>
       <c r="F75" s="33"/>
       <c r="G75" s="2"/>
@@ -2248,7 +2248,7 @@
         <v>186</v>
       </c>
       <c r="E76" s="43">
-        <v>1343</v>
+        <v>1363</v>
       </c>
       <c r="F76" s="33"/>
       <c r="G76" s="2"/>
@@ -2261,7 +2261,7 @@
         <v>187</v>
       </c>
       <c r="E77" s="64">
-        <v>5365</v>
+        <v>7327</v>
       </c>
       <c r="F77" s="33"/>
       <c r="G77" s="2"/>
@@ -3283,7 +3283,7 @@
         <v>130</v>
       </c>
       <c r="E155" s="43">
-        <v>12732</v>
+        <v>12962</v>
       </c>
       <c r="F155" s="33"/>
       <c r="G155" s="2"/>
@@ -3296,7 +3296,7 @@
         <v>131</v>
       </c>
       <c r="E156" s="43">
-        <v>8001</v>
+        <v>8041</v>
       </c>
       <c r="F156" s="33"/>
       <c r="G156" s="2"/>
@@ -4860,7 +4860,7 @@
         <v>55</v>
       </c>
       <c r="E276" s="43">
-        <v>12382</v>
+        <v>12392</v>
       </c>
       <c r="F276" s="33"/>
       <c r="G276" s="2"/>
@@ -4873,7 +4873,7 @@
         <v>56</v>
       </c>
       <c r="E277" s="43">
-        <v>11837</v>
+        <v>11847</v>
       </c>
       <c r="F277" s="33"/>
       <c r="G277" s="2"/>
@@ -4938,7 +4938,7 @@
         <v>61</v>
       </c>
       <c r="E282" s="43">
-        <v>7193</v>
+        <v>7223</v>
       </c>
       <c r="F282" s="33"/>
       <c r="G282" s="2"/>
@@ -5016,7 +5016,7 @@
         <v>67</v>
       </c>
       <c r="E288" s="43">
-        <v>9466</v>
+        <v>9474</v>
       </c>
       <c r="F288" s="33"/>
       <c r="G288" s="2"/>
@@ -5042,7 +5042,7 @@
         <v>69</v>
       </c>
       <c r="E290" s="43">
-        <v>2258</v>
+        <v>2268</v>
       </c>
       <c r="F290" s="33"/>
       <c r="G290" s="2"/>
@@ -5055,7 +5055,7 @@
         <v>70</v>
       </c>
       <c r="E291" s="43">
-        <v>3597</v>
+        <v>4337</v>
       </c>
       <c r="F291" s="33"/>
       <c r="G291" s="2"/>
@@ -5068,7 +5068,7 @@
         <v>71</v>
       </c>
       <c r="E292" s="43">
-        <v>6029</v>
+        <v>6072</v>
       </c>
       <c r="F292" s="33"/>
       <c r="G292" s="2"/>
@@ -5094,7 +5094,7 @@
         <v>73</v>
       </c>
       <c r="E294" s="43">
-        <v>2473</v>
+        <v>2778</v>
       </c>
       <c r="F294" s="33"/>
       <c r="G294" s="2"/>
@@ -5107,7 +5107,7 @@
         <v>74</v>
       </c>
       <c r="E295" s="43">
-        <v>2384</v>
+        <v>2534</v>
       </c>
       <c r="F295" s="33"/>
       <c r="G295" s="2"/>
@@ -5120,7 +5120,7 @@
         <v>75</v>
       </c>
       <c r="E296" s="43">
-        <v>3272</v>
+        <v>3480</v>
       </c>
       <c r="F296" s="33"/>
       <c r="G296" s="2"/>
@@ -5133,7 +5133,7 @@
         <v>76</v>
       </c>
       <c r="E297" s="43">
-        <v>2980</v>
+        <v>3036</v>
       </c>
       <c r="F297" s="33"/>
       <c r="G297" s="2"/>
@@ -5159,7 +5159,7 @@
         <v>78</v>
       </c>
       <c r="E299" s="43">
-        <v>3011</v>
+        <v>3021</v>
       </c>
       <c r="F299" s="33"/>
       <c r="G299" s="2"/>
@@ -5289,7 +5289,7 @@
         <v>88</v>
       </c>
       <c r="E309" s="43">
-        <v>342</v>
+        <v>352</v>
       </c>
       <c r="F309" s="33"/>
       <c r="G309" s="2"/>
@@ -5302,7 +5302,7 @@
         <v>89</v>
       </c>
       <c r="E310" s="43">
-        <v>573</v>
+        <v>586</v>
       </c>
       <c r="F310" s="33"/>
       <c r="G310" s="2"/>
@@ -7310,7 +7310,7 @@
   <phoneticPr fontId="5"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="64" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="356" max="6" man="1"/>
   </rowBreaks>

</xml_diff>